<commit_message>
Ajout de questions au fichier Excel
</commit_message>
<xml_diff>
--- a/TFP_APS_Questions_QCU_Reel_2025.xlsx
+++ b/TFP_APS_Questions_QCU_Reel_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://daher-my.sharepoint.com/personal/2104474_daher_com/Documents/Documents/WORK/PYTHON/apps/Questions_TFP_APS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="355" documentId="13_ncr:1_{2ACE7C71-CCF8-48B7-AEC7-69C3CEDFEA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15325C94-57E1-4052-A22A-E3F975B2DFE0}"/>
+  <xr:revisionPtr revIDLastSave="394" documentId="13_ncr:1_{2ACE7C71-CCF8-48B7-AEC7-69C3CEDFEA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CBEB89E-8F5C-4FAC-96A6-1B70A9A4549D}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste_Questions" sheetId="1" r:id="rId1"/>
@@ -18,31 +18,85 @@
     <sheet name="Feuil1" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_1h997plu2r3q" localSheetId="2">Feuil1!$A$169</definedName>
     <definedName name="_1x11d5k5io24" localSheetId="2">Feuil1!$A$26</definedName>
     <definedName name="_25b71xk2i301" localSheetId="2">Feuil1!$A$109</definedName>
     <definedName name="_2k99lr79hl9i" localSheetId="2">Feuil1!$A$5</definedName>
     <definedName name="_2utln1nfnqsx" localSheetId="2">Feuil1!$A$2</definedName>
+    <definedName name="_3bxdsxq7p8gw" localSheetId="2">Feuil1!$A$165</definedName>
+    <definedName name="_5ocrwot4q9or" localSheetId="2">Feuil1!$A$210</definedName>
     <definedName name="_62p8mewzupdh" localSheetId="2">Feuil1!$A$9</definedName>
+    <definedName name="_63ehbuvcc3tw" localSheetId="2">Feuil1!$A$174</definedName>
+    <definedName name="_6g3puvkrrskn" localSheetId="2">Feuil1!$A$173</definedName>
     <definedName name="_6sxpqe84lwy" localSheetId="2">Feuil1!$A$27</definedName>
+    <definedName name="_76u3b285zost" localSheetId="2">Feuil1!$A$191</definedName>
+    <definedName name="_76x8livz92e3" localSheetId="2">Feuil1!$A$207</definedName>
+    <definedName name="_7npq3rapq3b5" localSheetId="2">Feuil1!$A$211</definedName>
     <definedName name="_847vco2er5vx" localSheetId="2">Feuil1!#REF!</definedName>
+    <definedName name="_8i1gdydhdqo8" localSheetId="2">Feuil1!$A$206</definedName>
     <definedName name="_8vd2wc5v9auo" localSheetId="2">Feuil1!$A$12</definedName>
+    <definedName name="_92rzspumfy17" localSheetId="2">Feuil1!$A$204</definedName>
+    <definedName name="_9hexdyk5v0wx" localSheetId="2">Feuil1!$A$167</definedName>
+    <definedName name="_9jeesbxf4272" localSheetId="2">Feuil1!$A$193</definedName>
+    <definedName name="_9o8iqnw0882k" localSheetId="2">Feuil1!$A$181</definedName>
+    <definedName name="_a1blj5gc9j8j" localSheetId="2">Feuil1!$A$163</definedName>
+    <definedName name="_a20iajxrewtn" localSheetId="2">Feuil1!$A$212</definedName>
+    <definedName name="_a75ul79bzp21" localSheetId="2">Feuil1!$A$179</definedName>
     <definedName name="_atn6jtpgu1zu" localSheetId="2">Feuil1!$A$6</definedName>
+    <definedName name="_b77wlvmmh9wq" localSheetId="2">Feuil1!$A$176</definedName>
     <definedName name="_be1fc6ea00hk" localSheetId="2">Feuil1!$A$24</definedName>
+    <definedName name="_byzztlualq0q" localSheetId="2">Feuil1!$A$198</definedName>
+    <definedName name="_ccy2pemctn8p" localSheetId="2">Feuil1!$A$178</definedName>
+    <definedName name="_chgzqrac0okr" localSheetId="2">Feuil1!$A$161</definedName>
+    <definedName name="_dwwrsfcgojso" localSheetId="2">Feuil1!$A$171</definedName>
     <definedName name="_e8p5frs5ytai" localSheetId="2">Feuil1!$A$3</definedName>
     <definedName name="_eltq1ml39i8g" localSheetId="2">Feuil1!$A$110</definedName>
+    <definedName name="_f4und4vdlss2" localSheetId="2">Feuil1!$A$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Liste_Questions!$A$1:$J$76</definedName>
+    <definedName name="_g0y5qe76r34g" localSheetId="2">Feuil1!$A$195</definedName>
     <definedName name="_g70xgby2qf4" localSheetId="2">Feuil1!$A$4</definedName>
+    <definedName name="_g8ek9utgccwp" localSheetId="2">Feuil1!$A$209</definedName>
     <definedName name="_g9qmie434sne" localSheetId="2">Feuil1!$A$10</definedName>
+    <definedName name="_gawbf46ma6oj" localSheetId="2">Feuil1!$A$201</definedName>
+    <definedName name="_gelkcw7y8ynz" localSheetId="2">Feuil1!$A$199</definedName>
+    <definedName name="_hdt4xnw2zsex" localSheetId="2">Feuil1!$A$197</definedName>
+    <definedName name="_hm9eh7d297ex" localSheetId="2">Feuil1!$A$186</definedName>
     <definedName name="_hplm79wzz7gn" localSheetId="2">Feuil1!#REF!</definedName>
+    <definedName name="_i1nfs8unu8of" localSheetId="2">Feuil1!$A$185</definedName>
     <definedName name="_i84ik2pub0j3" localSheetId="2">Feuil1!$A$23</definedName>
+    <definedName name="_ieozcmlv3r2" localSheetId="2">Feuil1!$A$184</definedName>
+    <definedName name="_iqeveq8of09t" localSheetId="2">Feuil1!$A$168</definedName>
+    <definedName name="_j9lo7fkxjlb" localSheetId="2">Feuil1!$A$160</definedName>
+    <definedName name="_kc00q4gy8hb8" localSheetId="2">Feuil1!$A$183</definedName>
+    <definedName name="_kg2jlon5v06" localSheetId="2">Feuil1!$A$192</definedName>
+    <definedName name="_kor4i06yw3hg" localSheetId="2">Feuil1!$A$190</definedName>
+    <definedName name="_kwnngch1lt48" localSheetId="2">Feuil1!$A$196</definedName>
+    <definedName name="_lx174ek5g80a" localSheetId="2">Feuil1!$A$200</definedName>
     <definedName name="_nyqwx0jkl5qi" localSheetId="2">Feuil1!$A$33</definedName>
+    <definedName name="_nz347gkbav67" localSheetId="2">Feuil1!$A$180</definedName>
+    <definedName name="_odb06e873shv" localSheetId="2">Feuil1!$A$182</definedName>
     <definedName name="_p9wiu4shs9hc" localSheetId="2">Feuil1!$A$112</definedName>
+    <definedName name="_pzw7706yg5ao" localSheetId="2">Feuil1!$A$162</definedName>
+    <definedName name="_qf459c9a8pp1" localSheetId="2">Feuil1!$A$194</definedName>
+    <definedName name="_qxb3o5v8mgjr" localSheetId="2">Feuil1!$A$172</definedName>
+    <definedName name="_r9s9ghg1e3hf" localSheetId="2">Feuil1!$A$189</definedName>
+    <definedName name="_sicn53eiffia" localSheetId="2">Feuil1!$A$166</definedName>
     <definedName name="_tt764b9auzq8" localSheetId="2">Feuil1!$A$8</definedName>
+    <definedName name="_u74njex1xmue" localSheetId="2">Feuil1!$A$202</definedName>
     <definedName name="_u9haniwxsi9j" localSheetId="2">Feuil1!$A$16</definedName>
+    <definedName name="_utuurwq44qbd" localSheetId="2">Feuil1!$A$214</definedName>
+    <definedName name="_v2a1uzdymhjv" localSheetId="2">Feuil1!$A$205</definedName>
+    <definedName name="_vdgtxnft4z9o" localSheetId="2">Feuil1!$A$164</definedName>
     <definedName name="_vk618iff2ee1" localSheetId="2">Feuil1!$A$111</definedName>
+    <definedName name="_vs7np853i52g" localSheetId="2">Feuil1!$A$177</definedName>
+    <definedName name="_vyvwb23eh5z1" localSheetId="2">Feuil1!$A$208</definedName>
+    <definedName name="_w3sb88kffkq" localSheetId="2">Feuil1!$A$213</definedName>
     <definedName name="_wpn81467iw0b" localSheetId="2">Feuil1!$A$7</definedName>
+    <definedName name="_x6nck1a900y" localSheetId="2">Feuil1!$A$187</definedName>
     <definedName name="_xgrsy6hezdp9" localSheetId="2">Feuil1!$A$25</definedName>
+    <definedName name="_y4xt3quxwyvi" localSheetId="2">Feuil1!$A$175</definedName>
     <definedName name="_yj4hh6ff2wx9" localSheetId="2">Feuil1!$A$28</definedName>
+    <definedName name="_yyxysi2ip7um" localSheetId="2">Feuil1!$A$203</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -84,7 +138,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2037" uniqueCount="1200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2592" uniqueCount="1507">
   <si>
     <t>UV</t>
   </si>
@@ -5457,12 +5511,933 @@
   <si>
     <t>Les travaux concernent la coactivité sur les chantiers de bâtiment et de génie civil</t>
   </si>
+  <si>
+    <t>1 - [UV7] Que signifie le R de N.R.B.C-E ?|Radiologique|Radicalisé|Radioactif|Aucune des autres réponses|Rayonnant|A</t>
+  </si>
+  <si>
+    <t>2 - [UV7] Le Pneumothorax peut être occasionné par :|Toutes les réponses sont bonnes|Une explosion (Blast primaire)|Une perforation par une côte|Une plaie pénétrante par arme blanche|Une plaie pénétrante par balle|A</t>
+  </si>
+  <si>
+    <t>3 - [UV7] Parmi ces infractions, laquelle porte atteinte aux intérêts fondamentaux de la nation ?|La délation|L’abus de droit public|La rébellion|Le sabotage|La violation de domicile|D</t>
+  </si>
+  <si>
+    <t>4 - [UV7] Dans le cadre d’un risque d’attentat, que peut faire le Préfet ?|Décréter l’état d’urgence, mais seulement au niveau “vigilance”|Faire procéder à des fouilles à corps par des ASP|Accroître les contrôles aux frontières|Aucune des autres réponses|Interdire la circulation, instaurer un couvre-feu et limiter les allées/venues des personnes|E</t>
+  </si>
+  <si>
+    <t>5 - [UV7] Témoin direct d’un attentat en cours sur votre site, quelles consignes à suivre sont les plus appropriées ?|Alerter les personnes autour de vous|Si possible, aider les autres personnes à s’échapper|Laisser vos affaires derrière vous|Si vous ne pouvez pas courir, se confiner, éteindre la lumière et couper le son des appareils à proximité|Toutes les réponses précédentes sont exactes|E</t>
+  </si>
+  <si>
+    <t>6 - [UV11] Un groupe d’individus cagoulés et armés pénètre dans votre établissement et vous êtes seul : que faites-vous ?|J’appelle la relève pour me venir en aide le plus tôt possible|Je m’enfuis et je fais appel aux forces de l’ordre le plus rapidement possible|Je m’enfuis si je peux ou sinon je me confine, et je contacte le 114 par sms|Aucune des autres réponses|Je dois agir physiquement pour les expulser de l’établissement|C</t>
+  </si>
+  <si>
+    <t>7 - [UV9] Un agent de prévention et de sécurité a-t-il le droit de pratiquer des palpations de sécurité lors de manifestations sportives, récréatives ou culturelles ?|Oui, en toutes circonstances|Oui, s’il est habilité par son entreprise|Non, sauf s’il est habilité par son employeur|Aucune des autres réponses|Oui, si la manifestation dépasse 300 personnes et sous le contrôle d’un OPJ et que la personne palpée soit du même sexe que l’agent de sécurité|E</t>
+  </si>
+  <si>
+    <t>8 - [UV9] Je suis agent dans un établissement : sous quelles conditions ai-je le droit d’inspecter des sacs ?|Je peux faire une inspection visuelle même si ce n’est pas dans les consignes|Aucune des autres réponses|Si c’est prévu dans les consignes, je peux fouiller les sacs sans avoir besoin du consentement du propriétaire|J’ai le droit de faire une inspection visuelle des bagages et, avec le consentement de leur propriétaire, à leur fouille|Je peux vérifier visuellement et fouiller tous les sacs|D</t>
+  </si>
+  <si>
+    <t>9 - [UV11] En cas de détection incendie, sur quelle unité le voyant est-il lumineux ?|D.A.S.|C.M.S.I.|S.M.S.I.|S.D.I.|Aucune des réponses précédentes|D</t>
+  </si>
+  <si>
+    <t>10 - [UV7] Que dois-je regarder pour détecter un potentiel terroriste ?|Son comportement|La pratique de sa religion|Aucune des autres réponses|Ses antécédents judiciaires|Son apparence physique|A</t>
+  </si>
+  <si>
+    <t>11 - [UV7] Qu’est-ce que la zone d’exclusion dans un périmètre de sécurité immédiat ?|La zone de prise en charge par les secours|La zone de danger et d’intervention|La zone de commandement des forces de l’ordre|Aucune des autres réponses|La zone d’accueil des force de l’ordre et des secours|B</t>
+  </si>
+  <si>
+    <t>12 - [UV2] Un revolver chambré pour le calibre 38 spécial est une arme de catégorie :|C|D|A|Aucune des autres réponses|B|B</t>
+  </si>
+  <si>
+    <t>13 - [UV2] Le vol avec arme est qualifié de :|Crime terroriste|Aucune des autres réponses|Délit qualifié|Délit aggravé|Crime|E</t>
+  </si>
+  <si>
+    <t>14 - [UV12] Lorsque des véhicules sont susceptibles de pénétrer au sein de périmètre de protection (L266-1 du CSI), la loi peut également en subordonner l’accès à l’inspection visuelle du contenu du véhicule :|Sans le consentement de son conducteur, par un agent de prévention et de sécurité|Sans le consentement de son conducteur, par un agent de prévention et de sécurité mais sous le contrôle d’un OPJ|Avec le consentement de son conducteur, par un agent de prévention et de sécurité|Avec le consentement de son conducteur, par un agent de prévention et de sécurité placé sous l’autorité d’un OPJ|Aucune des autres réponses|E</t>
+  </si>
+  <si>
+    <t>15 - [UV12] Le fait d’accéder frauduleusement à des données informatiques issues d’images de vidéosurveillance constitue l’infraction de :|Atteinte au système de traitement automatisé de données|Entrave à la libre circulation des données|Dégradation ou détérioration d’un système de traitement de données informatiques |Aucune des autres réponses|Vol de données informatiques|A</t>
+  </si>
+  <si>
+    <t>16 - [UV12] Que signifie l’acronyme P.I.F. dans le cadre d’un système de sécurité lors d’un événement ?|Point ou Poste d’Inspection Filtrage|Poste Itinérant de Filtrage|Passage Interdit à la Foule|Aucune des autres réponses|Permis d’Inspection et de Fouille|A</t>
+  </si>
+  <si>
+    <t>17 - [UV12] Le plan ORSEC est :|Aucune des autres réponses|Un plan de limitation des déplacements dans le cadre du plan Vigipirates “Urgence Attentat”|Un plan d’Organisation de la Réponses de la Sécurité Civile|Un plan de circulation des riverains lors des événement culturels ou festifs|Un plan d’intervention coordonné des forces de l’ordre publiques et privées|C</t>
+  </si>
+  <si>
+    <t>18 - [UV8] Suite à un vol dans un magasin, le chef de poste du PCS reçoit les forces de l’ordre et il peut déposer plainte :|Non, car c’est du ressort exclusif d’un responsable du magasin habilité|Oui, seulement en l’absence du responsable du magasin|Aucune des autres réponses|Oui, car il est le chef de poste et il est donc habilité à déposer plainte|Oui, s’il a l’accord du responsable du magasin|A</t>
+  </si>
+  <si>
+    <t>19 - [UV8] Une zone de protection périphérique concerne :|Un objet précis|Aucune des autres réponses|Un local|Une vitrine|Une clôture|E</t>
+  </si>
+  <si>
+    <t>20 - [UV8] Une zone de protection ponctuelle concerne :|Un local|Aucune des autres réponses|Une vitrine|Une clôture|Un objet précis|E</t>
+  </si>
+  <si>
+    <t>21 - [UV8] Les convoyeurs de fonds peuvent-ils être armés lorsqu’ils effectuent en véhicule banalisé un transport de fonds, bijoux ou métaux précieux ?|Oui, avec l’autorisation du Préfet|Non, ils ne peuvent pas être armés|Oui, si la valeur des biens est supérieure à 1,3 millions d’euros|Aucune des autres réponses|Oui sur ordre de la société|B</t>
+  </si>
+  <si>
+    <t>22 - [UV7] Que signifie NRBC-E ?|Nationaliste-Radiologique-Bactériologique-Cyberterrorisme et Explosive|Nucléaire-Radiologique-Biologique-Chimique et Explosive|Nucléaire-Radiotechnologique-Bactériologique-Catastrophique et Explosive|Nationaliste-Régionaliste-Bracage-Contrôle et Enlèvement|Aucune des autres réponses|B</t>
+  </si>
+  <si>
+    <t>23 - [UV7] En cas de plan Vigipirate, l’accès à n’importe quel établissement peut être soumis à une palpation de sécurité : qui peut en décider ?|Le Préfet par un arrêté spécifique|L’agent de sécurité si les consignes spéciales le prévoyants|Le chef d’établissement dans son règlement intérieur|Le CNAPS par une circulaire ministérielle|Aucune des autres réponses|A</t>
+  </si>
+  <si>
+    <t>24 - [UV7] Qu’est-ce que l’état d’urgence ?|Un régime exceptionnel qui permet à l’Etat français de gérer une crise|Un régime qui donne des pouvoirs supplémentaires aux agents de prévention et de sécurité|Un régime continu servant à instaurer un climat de sécurité au peuple|Un régime totalitaire qui octroie les pleins pouvoirs au Président de la République|Aucune des autres réponses|A</t>
+  </si>
+  <si>
+    <t>25 - [UV7] Suite à une blessure par balle sur le torse d’une victime, comment puis-je la secourir sans provoquer un pneumothorax ?|Aucune des autres réponses|En posant dès que possible un garrot|En réalisant un pansement 3 côtés|En bouchant le trou formé par l’impact avec ma main|En mettant en place la réanimation cardio-pulmonaire|C</t>
+  </si>
+  <si>
+    <t>26 - [UV7] Quelles sont les grandes priorités de réaction que je dois adopter face à une attaque terroriste ?|Courir, m'enfermer, appeler, attaquer si nécessaire|M’échapper, me cacher, secourir, combattre systématiquement|Alerter, éteindre, méloigner, boxer|Aucune des autres réponses|A</t>
+  </si>
+  <si>
+    <t>27 - [UV7] Qu’est-ce que le terrorisme d’Etat ?|Aucune des autres réponses|Lorsqu’un peuple terrorise son gouvernement|Lorsqu’un Etat terrorise son peuple|Lorsqu’un Etat combat de le terrorisme à l’intérieur de ses frontières|Lorsqu’une organisation terroriste veut prendre le pouvoir d’un Etat|C</t>
+  </si>
+  <si>
+    <t>28 - [UV2] Un agent de sécurité exerçant ses fonctions dans un parc d’attraction peut-il appréhender un individu qui y entre avec une matraque et tente d’agresser un salarié du parc ?|Il peut juste l’aborder mais il ne peut pas l’appréhender en vertu de l’art. 73 du CPP|Aucune des autres réponses|Oui, car il sera dans le cadre de l’état de nécessité prévu dans l’art. 121-2 du Code Pénal|Non, car il n’y a pas d’infraction prévue pour ce type de fait|Le port d’une matraque constituant un délit, il peut appréhender l’individu au titre de l’art. 73 du CPP|E</t>
+  </si>
+  <si>
+    <t>29 - [UV2] Un agent de sécurité privé peut être sanctionné par le CNAPS :|À une pénalité financière mais sans limite prise en charge par l’entreprise|À aucune pénalité financière|À une pénalité financière allant jusqu’à 10 000 euros|À une pénalité financière allant jusqu’à 7 500 euros|À une pénalité financière inférieure à 1 500 euros|D</t>
+  </si>
+  <si>
+    <t>30 - [UV12] À quoi peut servir un PPI/POI/PER ?|Aucune des autres réponses|À coordonner les moyens internes des installations classées|À prévoir la mobilisation des services de secours publics|À protéger les installations recevant du public|À planifier les opérations de maintien de l’ordre|C</t>
+  </si>
+  <si>
+    <t>31 - [UV12] Il est puni par le code du sport (L332-3) dans une enceinte sportive, lors du déroulement ou de la retransmission en public d’une manifestation sportive :|Le fait d’introduire ou de tenter d’introduire, par force ou par fraude, des boissons alcoolisées|Toutes les réponses sont exactes|Le fait d’avoir, en état d’ivresse, pénétré ou tenté de pénétrer par force ou par fraude|D’un an d’emprisonnement ou d’amende|Le fait d’accéder en état d’ivresse|A</t>
+  </si>
+  <si>
+    <t>32 - [UV12] Les organisateurs de manifestations sportives, récréatives ou culturelles sont tenus (R211-22 du CSI) :|D’en faire la déclaration uniquement si elles sont sur la liste des événements exposés|D’en faire la déclaration au Préfet de région au moins un an avant l’événement|D’en faire la déclaration aux maires ou aux Préfets de police, si la manifestation peut atteindre plus de 1500 personnes|Aucune des autres réponses|D’en faire la déclaration aux maires si la manifestation peut atteindre plus de 300 personnes et aux Préfets si elle dépasse plus de 1500 personnes|C</t>
+  </si>
+  <si>
+    <t>33 - [UV9] Je suis agent dans un magasin : sous quelles conditions ai-je le droit d’inspecter des sacs ?|Je peux faire une inspection visuelle, dès lors que j’ai un doute|Je peux vérifier visuellement et fouiller les sacs sans avoir besoin du consentement du propriétaire|Aucune des autres réponses|J’ai le droit de faire une inspection visuelle des bagages et, avec le consentement de leur propriétaire, à leur fouille|Si c’est prévu dans les consignes, je peux vérifier visuellement et fouiller les sacs sans avoir besoin du consentement du propriétaires|D</t>
+  </si>
+  <si>
+    <t>34 - [UV8] Qu’est-ce qu’une zone de protection ?|Lieu protégé par des filets empêchant l’introduction de pigeons dans le site|Lieu protégé par des paroies possédant une isolation phonique|Aucune des autres réponses|Lieu protégé contre les intempéries|Lieu protégé par un obstacle s’opposant à pénétration d’intrus dans le site|E</t>
+  </si>
+  <si>
+    <t>35 - [UV8] Un point dit vulnérable lors d’une ronde est :|Un point comportant un danger permanent|Un point qui en cas d’atteinte pourrait handicaper le bon fonctionnement de l’entreprise|Un point régulièrement mis en défaut|Aucune des autres réponses|Un point sensible convoité par les voleurs|B</t>
+  </si>
+  <si>
+    <t>36 - [UV8] Pendant votre ronde, vous découvrez un local en désordre avec un pied de biche au sol. Que faites-vous ?|Vous ramassez le pied de biche afin d’avoir un objet pour vous défendre|Vous prévenez immédiatement le PCS et inspecter prudemment les locaux voisins|Aucune des autres réponses|Vous ne faites rien et continuez votre rondre, c’est sûrement le bureau d’un salarié désordonné|Vous refermez la porte et prévenez le PCS|B</t>
+  </si>
+  <si>
+    <t>37 - [UV6] Un agent de sécurité privé masculin doit appréhender un voleur en sortie de caisse, mais il s’agit d’une femme :|Il doit appeler une collègue du même sexe|Il agit normalement, néanmoins il est conseillé d’appeler un témoin féminin|Aucune des autres réponses|Il doit demander l’autorisation de la personne|Il ne peut rien faire sur une personne de sexe opposé|B</t>
+  </si>
+  <si>
+    <t>38 - [UV2] Les agents de sécurité employés par un bailleur d’immeuble à usage d’habitations peuvent être armés :|D’un bâton de défense de type TONFA|D’un fusil à pompe|D’une grenade lacrymogène ayant une capacité inférieure à 100 ml|Aucune des autres réponses|D’un pistolet mitrailleur|A</t>
+  </si>
+  <si>
+    <t>39 - [UV12] Le schéma d’installation de la vidéoprotection permet :|D’installer, de maintenir et de mettre à disposition des prestataires des images|De capter, de transmettre, de stocker, de visionner les images|Aucune des autres réponses|De garantir aux forces de l’ordre la bonne réalisation de la mission de sûreté|De compléter le système de surveillance incendie|B</t>
+  </si>
+  <si>
+    <t>40 - [UV12] À quoi correspond une crash barrière ?|Aucune des autres réponses|Un système de barrière type passage à niveau pour bloquer les accès|Des barrières de sécurité équipés de pieds empêchant le renversement|Un test en laboratoire de la résistance des barrières|L’action de lancer des barrières sur des véhicules voulant forcer l’accès|C</t>
+  </si>
+  <si>
+    <t>41 - [UV12] Un APS effectue une ronde dans la chaufferie gaz, il peut y entrer si :|Il dispose d’une radio fabriquée après le 1er juillet 2017|Il dispose d’un matériel anti-déflagrant|Il dispose d’un émetteur multi-fréquences|Il dispose d’une pastille de détection de gaz homologuée|Aucune des autres réponses|B</t>
+  </si>
+  <si>
+    <t>42 - [UV11] Sur votre GTB/GTC vous recevez une alarme SURCHAUFF au niveau de la chaufferie. Que devez-vous faire en premier ?|Aucune des autres réponses|Arrêter le signal sonore de l’alarme|Appeler les services de secours|Couper la chaudière|Appeler le technicien compétent|B</t>
+  </si>
+  <si>
+    <t>43 - [UV11] En vous rendant sur une levée de doute intrusion, votre PC vous appelle car une détection incendie vient d’avoir lieu. Que faites-vous ?|Je termine la levée de doute intrusion sans effectuer les contrôles de rigueur pour aller sur la levée de doute incendie|Je fais demi-tour et priorise la détection incendie dont la gravité peut être supérieure|Aucune des autres réponses|Je poursuis la levée de doute intrusion, étant presque arrivé|Je demande au chef de poste d’effectuer lui-même la levée de doute incendie|B</t>
+  </si>
+  <si>
+    <t>44 - [UV11] En cas d’alarme observée sur la centrale incendie, quelle est généralement la procédure à suivre ?|Appel de l’astreinte incendie, attente des secours, intervention éventuelle sur le feu|Acquittement du signal sonore, lecture de l’information, levée de doute, plan d’action conforme aux consignes du site|Aucune des autres réponses|Levée de doute, appel des secours, retour au PCS|Intervention immédiate sur feu, appel des secours, réinitialisation central incendie|B</t>
+  </si>
+  <si>
+    <t>45 - [UV9] Quelles sont les méthodes pour les agents masculins pour effectuer des vérifications de sécurité sur des femmes qui sont au contrôle d’accès :|Les palpations de sécurité|La fouille à corps uniquement avec le consentement de la personne|La fouille au corps|Aucune des autres réponses|Le contrôle visuel des bagages|E</t>
+  </si>
+  <si>
+    <t>46 - [UV9] Dans quelle situation puis-je effectuer des palpations de sécurité ?|Dans tout le magasin sur des personnes soupçonnées de vouloir fumer|À l’intérieur d’une salle de concert à la demande du chef de poste|Dans tout lieu visé par un arrêté préfectoral|À la sortie du magasin sur un individu connu pour des actes de vol|Aucune des autres réponses|C</t>
+  </si>
+  <si>
+    <t>47 - [UV8] Certaines circonstances peuvent aggraver le vol. Par exemple quand le vol est commis :|Par plusieurs personnes|Chez une personne dépositaire de l’autorité publique|Sur une personne dans la journée|Aucune des autres réponses|Dans un local sous surveillance électronique|A</t>
+  </si>
+  <si>
+    <t>48 - [UV7] Dès l’arrivée des forces de l’ordre, dans une zone d’attentat, vous devez en premier :|Leur parler de la situation|Courir vers eux|Leur indiquer l’emplacement des victimes|Suivre leurs instructions|Aucune des autres réponses|D</t>
+  </si>
+  <si>
+    <t>49 - [UV7] Parmi les types de “BLAST” suivants, lequel ou lesquels existent ?|BLAST primaire|BLAST tertiaire|BLAST quaternaire|Toutes les réponses précédentes sont exactes|BLAST secondaire|D</t>
+  </si>
+  <si>
+    <t>50 - [UV2] Agent de sécurité, je dispose d’un véhicule d’entreprise équipé d’un gyrophare orange :|Aucune des autres réponses|C’est absolument interdit|C’est autorisé uniquement à l’intérieur des sites surveillés, si les consignes le prévoient|Seuls les gyrophares bleus sont autorisés pour les agents de sécurité|C’est interdit, sauf en situation d’urgence attentat|C</t>
+  </si>
+  <si>
+    <t>51 - [UV2] Selon la loi, est une arme par destination :|Tout objet conçu pour usage professionnel|Tout objet conçu pour tuer ou blesser|Aucune des autres réponses|Tout objet susceptible de présenter un danger pour des personnes, dès lors qu’il est utilisé pour menacer|Tout objet pouvant causer des dommages|D</t>
+  </si>
+  <si>
+    <t>52 - [UV11] Le report d’alarme d’une centrale intrusion est un dispositif :|Uniquement destiné aux équipes de sûreté en cas d’intrusion|De secours en cas de défaillance du clavier principal|Qui permet aux agents d’accéder à certaines informations hors du PCS|De cloisonnement anti-intrusion indépendant du système central|Aucune des autres réponses|C</t>
+  </si>
+  <si>
+    <t>53 - [UV14] Dans quel document l’APS peut trouver les mesures opératoires des secours extérieurs lors d’un sinistre majeur ?|Le Plan des Opérations Externes (P.O.E.)|Le Plan Particulier d’Intervention (P.P.I. ou équivalent)|Le Plan de Secours Extérieurs (P.S.E.)|Le Plan Particulier des Risques Majeurs (P.P.R.M.)|Aucune des autres réponses|B</t>
+  </si>
+  <si>
+    <t>54 - [UV14] Quand doit-on rédiger notamment impérativement un Plan de Prévention ?|En cas de travaux dangereux listés dans l’arrêté du 19 mars 1993|Uniquement lorsque les consignes de sûreté le prévoient|Si vous estimez que l’importance des travaux le nécessitent|Uniquement sur demande explicite du client|Aucune des autres réponses|A</t>
+  </si>
+  <si>
+    <t>55 - [UV14] Quel est l’objectif général de la prévention ?|Définir les mesures de sûreté|Protéger l’employeur du risque pénal|Améliorer les statistiques concernant les taux d’accidents|Éviter ou limiter les dommages|Aucune des autres réponses|D</t>
+  </si>
+  <si>
+    <t>Radiologique</t>
+  </si>
+  <si>
+    <t>Radicalisé</t>
+  </si>
+  <si>
+    <t>Radioactif</t>
+  </si>
+  <si>
+    <t>Rayonnant</t>
+  </si>
+  <si>
+    <t>[UV7] Le Pneumothorax peut être occasionné par :</t>
+  </si>
+  <si>
+    <t>Une explosion (Blast primaire)</t>
+  </si>
+  <si>
+    <t>Une perforation par une côte</t>
+  </si>
+  <si>
+    <t>Une plaie pénétrante par arme blanche</t>
+  </si>
+  <si>
+    <t>Une plaie pénétrante par balle</t>
+  </si>
+  <si>
+    <t>[UV7] Parmi ces infractions, laquelle porte atteinte aux intérêts fondamentaux de la nation ?</t>
+  </si>
+  <si>
+    <t>La délation</t>
+  </si>
+  <si>
+    <t>L’abus de droit public</t>
+  </si>
+  <si>
+    <t>La rébellion</t>
+  </si>
+  <si>
+    <t>Le sabotage</t>
+  </si>
+  <si>
+    <t>La violation de domicile</t>
+  </si>
+  <si>
+    <t>[UV7] Dans le cadre d’un risque d’attentat, que peut faire le Préfet ?</t>
+  </si>
+  <si>
+    <t>Décréter l’état d’urgence, mais seulement au niveau “vigilance”</t>
+  </si>
+  <si>
+    <t>Faire procéder à des fouilles à corps par des ASP</t>
+  </si>
+  <si>
+    <t>Accroître les contrôles aux frontières</t>
+  </si>
+  <si>
+    <t>Interdire la circulation, instaurer un couvre-feu et limiter les allées/venues des personnes</t>
+  </si>
+  <si>
+    <t>[UV7] Témoin direct d’un attentat en cours sur votre site, quelles consignes à suivre sont les plus appropriées ?</t>
+  </si>
+  <si>
+    <t>Alerter les personnes autour de vous</t>
+  </si>
+  <si>
+    <t>Si possible, aider les autres personnes à s’échapper</t>
+  </si>
+  <si>
+    <t>Laisser vos affaires derrière vous</t>
+  </si>
+  <si>
+    <t>Si vous ne pouvez pas courir, se confiner, éteindre la lumière et couper le son des appareils à proximité</t>
+  </si>
+  <si>
+    <t>[UV11] Un groupe d’individus cagoulés et armés pénètre dans votre établissement et vous êtes seul : que faites-vous ?</t>
+  </si>
+  <si>
+    <t>J’appelle la relève pour me venir en aide le plus tôt possible</t>
+  </si>
+  <si>
+    <t>Je m’enfuis et je fais appel aux forces de l’ordre le plus rapidement possible</t>
+  </si>
+  <si>
+    <t>Je m’enfuis si je peux ou sinon je me confine, et je contacte le 114 par sms</t>
+  </si>
+  <si>
+    <t>Je dois agir physiquement pour les expulser de l’établissement</t>
+  </si>
+  <si>
+    <t>[UV9] Un agent de prévention et de sécurité a-t-il le droit de pratiquer des palpations de sécurité lors de manifestations sportives, récréatives ou culturelles ?</t>
+  </si>
+  <si>
+    <t>Oui, en toutes circonstances</t>
+  </si>
+  <si>
+    <t>Oui, s’il est habilité par son entreprise</t>
+  </si>
+  <si>
+    <t>Non, sauf s’il est habilité par son employeur</t>
+  </si>
+  <si>
+    <t>Oui, si la manifestation dépasse 300 personnes et sous le contrôle d’un OPJ et que la personne palpée soit du même sexe que l’agent de sécurité</t>
+  </si>
+  <si>
+    <t>[UV9] Je suis agent dans un établissement : sous quelles conditions ai-je le droit d’inspecter des sacs ?</t>
+  </si>
+  <si>
+    <t>Je peux faire une inspection visuelle même si ce n’est pas dans les consignes</t>
+  </si>
+  <si>
+    <t>Si c’est prévu dans les consignes, je peux fouiller les sacs sans avoir besoin du consentement du propriétaire</t>
+  </si>
+  <si>
+    <t>J’ai le droit de faire une inspection visuelle des bagages et, avec le consentement de leur propriétaire, à leur fouille</t>
+  </si>
+  <si>
+    <t>Je peux vérifier visuellement et fouiller tous les sacs</t>
+  </si>
+  <si>
+    <t>[UV11] En cas de détection incendie, sur quelle unité le voyant est-il lumineux ?</t>
+  </si>
+  <si>
+    <t>D.A.S.</t>
+  </si>
+  <si>
+    <t>C.M.S.I.</t>
+  </si>
+  <si>
+    <t>S.M.S.I.</t>
+  </si>
+  <si>
+    <t>S.D.I.</t>
+  </si>
+  <si>
+    <t>[UV7] Que dois-je regarder pour détecter un potentiel terroriste ?</t>
+  </si>
+  <si>
+    <t>Son comportement</t>
+  </si>
+  <si>
+    <t>La pratique de sa religion</t>
+  </si>
+  <si>
+    <t>Ses antécédents judiciaires</t>
+  </si>
+  <si>
+    <t>Son apparence physique</t>
+  </si>
+  <si>
+    <t>[UV7] Qu’est-ce que la zone d’exclusion dans un périmètre de sécurité immédiat ?</t>
+  </si>
+  <si>
+    <t>La zone de prise en charge par les secours</t>
+  </si>
+  <si>
+    <t>La zone de danger et d’intervention</t>
+  </si>
+  <si>
+    <t>La zone de commandement des forces de l’ordre</t>
+  </si>
+  <si>
+    <t>La zone d’accueil des force de l’ordre et des secours</t>
+  </si>
+  <si>
+    <t>[UV2] Un revolver chambré pour le calibre 38 spécial est une arme de catégorie :</t>
+  </si>
+  <si>
+    <t>[UV2] Le vol avec arme est qualifié de :</t>
+  </si>
+  <si>
+    <t>Crime terroriste</t>
+  </si>
+  <si>
+    <t>Délit qualifié</t>
+  </si>
+  <si>
+    <t>Délit aggravé</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>[UV12] Lorsque des véhicules sont susceptibles de pénétrer au sein de périmètre de protection (L266-1 du CSI), la loi peut également en subordonner l’accès à l’inspection visuelle du contenu du véhicule :</t>
+  </si>
+  <si>
+    <t>Avec le consentement de son conducteur, par un agent de prévention et de sécurité placé sous l’autorité d’un OPJ</t>
+  </si>
+  <si>
+    <t>[UV12] Le fait d’accéder frauduleusement à des données informatiques issues d’images de vidéosurveillance constitue l’infraction de :</t>
+  </si>
+  <si>
+    <t>Atteinte au système de traitement automatisé de données</t>
+  </si>
+  <si>
+    <t>Entrave à la libre circulation des données</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dégradation ou détérioration d’un système de traitement de données informatiques </t>
+  </si>
+  <si>
+    <t>[UV12] Que signifie l’acronyme P.I.F. dans le cadre d’un système de sécurité lors d’un événement ?</t>
+  </si>
+  <si>
+    <t>Point ou Poste d’Inspection Filtrage</t>
+  </si>
+  <si>
+    <t>Poste Itinérant de Filtrage</t>
+  </si>
+  <si>
+    <t>Passage Interdit à la Foule</t>
+  </si>
+  <si>
+    <t>Permis d’Inspection et de Fouille</t>
+  </si>
+  <si>
+    <t>[UV12] Le plan ORSEC est :</t>
+  </si>
+  <si>
+    <t>Un plan de limitation des déplacements dans le cadre du plan Vigipirates “Urgence Attentat”</t>
+  </si>
+  <si>
+    <t>Un plan d’Organisation de la Réponses de la Sécurité Civile</t>
+  </si>
+  <si>
+    <t>Un plan de circulation des riverains lors des événement culturels ou festifs</t>
+  </si>
+  <si>
+    <t>Un plan d’intervention coordonné des forces de l’ordre publiques et privées</t>
+  </si>
+  <si>
+    <t>[UV8] Suite à un vol dans un magasin, le chef de poste du PCS reçoit les forces de l’ordre et il peut déposer plainte :</t>
+  </si>
+  <si>
+    <t>Non, car c’est du ressort exclusif d’un responsable du magasin habilité</t>
+  </si>
+  <si>
+    <t>Oui, seulement en l’absence du responsable du magasin</t>
+  </si>
+  <si>
+    <t>Oui, car il est le chef de poste et il est donc habilité à déposer plainte</t>
+  </si>
+  <si>
+    <t>Oui, s’il a l’accord du responsable du magasin</t>
+  </si>
+  <si>
+    <t>[UV8] Une zone de protection périphérique concerne :</t>
+  </si>
+  <si>
+    <t>[UV8] Une zone de protection ponctuelle concerne :</t>
+  </si>
+  <si>
+    <t>[UV8] Les convoyeurs de fonds peuvent-ils être armés lorsqu’ils effectuent en véhicule banalisé un transport de fonds, bijoux ou métaux précieux ?</t>
+  </si>
+  <si>
+    <t>Oui, avec l’autorisation du Préfet</t>
+  </si>
+  <si>
+    <t>Non, ils ne peuvent pas être armés</t>
+  </si>
+  <si>
+    <t>Oui, si la valeur des biens est supérieure à 1,3 millions d’euros</t>
+  </si>
+  <si>
+    <t>Oui sur ordre de la société</t>
+  </si>
+  <si>
+    <t>[UV7] Que signifie NRBC-E ?</t>
+  </si>
+  <si>
+    <t>Nationaliste-Radiologique-Bactériologique-Cyberterrorisme et Explosive</t>
+  </si>
+  <si>
+    <t>Nucléaire-Radiologique-Biologique-Chimique et Explosive</t>
+  </si>
+  <si>
+    <t>Nucléaire-Radiotechnologique-Bactériologique-Catastrophique et Explosive</t>
+  </si>
+  <si>
+    <t>Nationaliste-Régionaliste-Bracage-Contrôle et Enlèvement</t>
+  </si>
+  <si>
+    <t>[UV7] En cas de plan Vigipirate, l’accès à n’importe quel établissement peut être soumis à une palpation de sécurité : qui peut en décider ?</t>
+  </si>
+  <si>
+    <t>Le Préfet par un arrêté spécifique</t>
+  </si>
+  <si>
+    <t>L’agent de sécurité si les consignes spéciales le prévoyants</t>
+  </si>
+  <si>
+    <t>Le chef d’établissement dans son règlement intérieur</t>
+  </si>
+  <si>
+    <t>Le CNAPS par une circulaire ministérielle</t>
+  </si>
+  <si>
+    <t>[UV7] Qu’est-ce que l’état d’urgence ?</t>
+  </si>
+  <si>
+    <t>Un régime exceptionnel qui permet à l’Etat français de gérer une crise</t>
+  </si>
+  <si>
+    <t>Un régime qui donne des pouvoirs supplémentaires aux agents de prévention et de sécurité</t>
+  </si>
+  <si>
+    <t>Un régime continu servant à instaurer un climat de sécurité au peuple</t>
+  </si>
+  <si>
+    <t>Un régime totalitaire qui octroie les pleins pouvoirs au Président de la République</t>
+  </si>
+  <si>
+    <t>[UV7] Suite à une blessure par balle sur le torse d’une victime, comment puis-je la secourir sans provoquer un pneumothorax ?</t>
+  </si>
+  <si>
+    <t>En posant dès que possible un garrot</t>
+  </si>
+  <si>
+    <t>En réalisant un pansement 3 côtés</t>
+  </si>
+  <si>
+    <t>En bouchant le trou formé par l’impact avec ma main</t>
+  </si>
+  <si>
+    <t>En mettant en place la réanimation cardio-pulmonaire</t>
+  </si>
+  <si>
+    <t>[UV7] Quelles sont les grandes priorités de réaction que je dois adopter face à une attaque terroriste ?</t>
+  </si>
+  <si>
+    <t>Courir, m'enfermer, appeler, attaquer si nécessaire</t>
+  </si>
+  <si>
+    <t>M’échapper, me cacher, secourir, combattre systématiquement</t>
+  </si>
+  <si>
+    <t>Alerter, éteindre, méloigner, boxer</t>
+  </si>
+  <si>
+    <t>[UV7] Qu’est-ce que le terrorisme d’Etat ?</t>
+  </si>
+  <si>
+    <t>Lorsqu’un peuple terrorise son gouvernement</t>
+  </si>
+  <si>
+    <t>Lorsqu’un Etat terrorise son peuple</t>
+  </si>
+  <si>
+    <t>Lorsqu’un Etat combat de le terrorisme à l’intérieur de ses frontières</t>
+  </si>
+  <si>
+    <t>Lorsqu’une organisation terroriste veut prendre le pouvoir d’un Etat</t>
+  </si>
+  <si>
+    <t>[UV2] Un agent de sécurité exerçant ses fonctions dans un parc d’attraction peut-il appréhender un individu qui y entre avec une matraque et tente d’agresser un salarié du parc ?</t>
+  </si>
+  <si>
+    <t>Il peut juste l’aborder mais il ne peut pas l’appréhender en vertu de l’art. 73 du CPP</t>
+  </si>
+  <si>
+    <t>Oui, car il sera dans le cadre de l’état de nécessité prévu dans l’art. 121-2 du Code Pénal</t>
+  </si>
+  <si>
+    <t>Non, car il n’y a pas d’infraction prévue pour ce type de fait</t>
+  </si>
+  <si>
+    <t>Le port d’une matraque constituant un délit, il peut appréhender l’individu au titre de l’art. 73 du CPP</t>
+  </si>
+  <si>
+    <t>[UV2] Un agent de sécurité privé peut être sanctionné par le CNAPS :</t>
+  </si>
+  <si>
+    <t>À une pénalité financière mais sans limite prise en charge par l’entreprise</t>
+  </si>
+  <si>
+    <t>À aucune pénalité financière</t>
+  </si>
+  <si>
+    <t>À une pénalité financière allant jusqu’à 10 000 euros</t>
+  </si>
+  <si>
+    <t>À une pénalité financière allant jusqu’à 7 500 euros</t>
+  </si>
+  <si>
+    <t>À une pénalité financière inférieure à 1 500 euros</t>
+  </si>
+  <si>
+    <t>[UV12] À quoi peut servir un PPI/POI/PER ?</t>
+  </si>
+  <si>
+    <t>À coordonner les moyens internes des installations classées</t>
+  </si>
+  <si>
+    <t>À prévoir la mobilisation des services de secours publics</t>
+  </si>
+  <si>
+    <t>À protéger les installations recevant du public</t>
+  </si>
+  <si>
+    <t>À planifier les opérations de maintien de l’ordre</t>
+  </si>
+  <si>
+    <t>[UV12] Il est puni par le code du sport (L332-3) dans une enceinte sportive, lors du déroulement ou de la retransmission en public d’une manifestation sportive :</t>
+  </si>
+  <si>
+    <t>Le fait d’introduire ou de tenter d’introduire, par force ou par fraude, des boissons alcoolisées</t>
+  </si>
+  <si>
+    <t>Le fait d’avoir, en état d’ivresse, pénétré ou tenté de pénétrer par force ou par fraude</t>
+  </si>
+  <si>
+    <t>D’un an d’emprisonnement ou d’amende</t>
+  </si>
+  <si>
+    <t>Le fait d’accéder en état d’ivresse</t>
+  </si>
+  <si>
+    <t>[UV12] Les organisateurs de manifestations sportives, récréatives ou culturelles sont tenus (R211-22 du CSI) :</t>
+  </si>
+  <si>
+    <t>D’en faire la déclaration au Préfet de région au moins un an avant l’événement</t>
+  </si>
+  <si>
+    <t>D’en faire la déclaration aux maires ou aux Préfets de police, si la manifestation peut atteindre plus de 1500 personnes</t>
+  </si>
+  <si>
+    <t>D’en faire la déclaration aux maires si la manifestation peut atteindre plus de 300 personnes et aux Préfets si elle dépasse plus de 1500 personnes</t>
+  </si>
+  <si>
+    <t>[UV9] Je suis agent dans un magasin : sous quelles conditions ai-je le droit d’inspecter des sacs ?</t>
+  </si>
+  <si>
+    <t>Je peux faire une inspection visuelle, dès lors que j’ai un doute</t>
+  </si>
+  <si>
+    <t>Je peux vérifier visuellement et fouiller les sacs sans avoir besoin du consentement du propriétaire</t>
+  </si>
+  <si>
+    <t>Si c’est prévu dans les consignes, je peux vérifier visuellement et fouiller les sacs sans avoir besoin du consentement du propriétaires</t>
+  </si>
+  <si>
+    <t>[UV8] Qu’est-ce qu’une zone de protection ?</t>
+  </si>
+  <si>
+    <t>Lieu protégé par des filets empêchant l’introduction de pigeons dans le site</t>
+  </si>
+  <si>
+    <t>Lieu protégé par des paroies possédant une isolation phonique</t>
+  </si>
+  <si>
+    <t>Lieu protégé contre les intempéries</t>
+  </si>
+  <si>
+    <t>Lieu protégé par un obstacle s’opposant à pénétration d’intrus dans le site</t>
+  </si>
+  <si>
+    <t>[UV8] Un point dit vulnérable lors d’une ronde est :</t>
+  </si>
+  <si>
+    <t>Un point régulièrement mis en défaut</t>
+  </si>
+  <si>
+    <t>Un point sensible convoité par les voleurs</t>
+  </si>
+  <si>
+    <t>[UV8] Pendant votre ronde, vous découvrez un local en désordre avec un pied de biche au sol. Que faites-vous ?</t>
+  </si>
+  <si>
+    <t>Vous ramassez le pied de biche afin d’avoir un objet pour vous défendre</t>
+  </si>
+  <si>
+    <t>Vous prévenez immédiatement le PCS et inspecter prudemment les locaux voisins</t>
+  </si>
+  <si>
+    <t>Vous ne faites rien et continuez votre rondre, c’est sûrement le bureau d’un salarié désordonné</t>
+  </si>
+  <si>
+    <t>Vous refermez la porte et prévenez le PCS</t>
+  </si>
+  <si>
+    <t>[UV6] Un agent de sécurité privé masculin doit appréhender un voleur en sortie de caisse, mais il s’agit d’une femme :</t>
+  </si>
+  <si>
+    <t>Il doit appeler une collègue du même sexe</t>
+  </si>
+  <si>
+    <t>Il agit normalement, néanmoins il est conseillé d’appeler un témoin féminin</t>
+  </si>
+  <si>
+    <t>Il doit demander l’autorisation de la personne</t>
+  </si>
+  <si>
+    <t>Il ne peut rien faire sur une personne de sexe opposé</t>
+  </si>
+  <si>
+    <t>[UV2] Les agents de sécurité employés par un bailleur d’immeuble à usage d’habitations peuvent être armés :</t>
+  </si>
+  <si>
+    <t>D’un fusil à pompe</t>
+  </si>
+  <si>
+    <t>D’une grenade lacrymogène ayant une capacité inférieure à 100 ml</t>
+  </si>
+  <si>
+    <t>D’un pistolet mitrailleur</t>
+  </si>
+  <si>
+    <t>[UV12] Le schéma d’installation de la vidéoprotection permet :</t>
+  </si>
+  <si>
+    <t>[UV12] À quoi correspond une crash barrière ?</t>
+  </si>
+  <si>
+    <t>Un système de barrière type passage à niveau pour bloquer les accès</t>
+  </si>
+  <si>
+    <t>Des barrières de sécurité équipés de pieds empêchant le renversement</t>
+  </si>
+  <si>
+    <t>Un test en laboratoire de la résistance des barrières</t>
+  </si>
+  <si>
+    <t>L’action de lancer des barrières sur des véhicules voulant forcer l’accès</t>
+  </si>
+  <si>
+    <t>[UV12] Un APS effectue une ronde dans la chaufferie gaz, il peut y entrer si :</t>
+  </si>
+  <si>
+    <t>Il dispose d’une radio fabriquée après le 1er juillet 2017</t>
+  </si>
+  <si>
+    <t>Il dispose d’un matériel anti-déflagrant</t>
+  </si>
+  <si>
+    <t>Il dispose d’un émetteur multi-fréquences</t>
+  </si>
+  <si>
+    <t>Il dispose d’une pastille de détection de gaz homologuée</t>
+  </si>
+  <si>
+    <t>[UV11] Sur votre GTB/GTC vous recevez une alarme SURCHAUFF au niveau de la chaufferie. Que devez-vous faire en premier ?</t>
+  </si>
+  <si>
+    <t>Arrêter le signal sonore de l’alarme</t>
+  </si>
+  <si>
+    <t>Appeler les services de secours</t>
+  </si>
+  <si>
+    <t>Couper la chaudière</t>
+  </si>
+  <si>
+    <t>Appeler le technicien compétent</t>
+  </si>
+  <si>
+    <t>[UV11] En vous rendant sur une levée de doute intrusion, votre PC vous appelle car une détection incendie vient d’avoir lieu. Que faites-vous ?</t>
+  </si>
+  <si>
+    <t>Je termine la levée de doute intrusion sans effectuer les contrôles de rigueur pour aller sur la levée de doute incendie</t>
+  </si>
+  <si>
+    <t>Je fais demi-tour et priorise la détection incendie dont la gravité peut être supérieure</t>
+  </si>
+  <si>
+    <t>Je poursuis la levée de doute intrusion, étant presque arrivé</t>
+  </si>
+  <si>
+    <t>Je demande au chef de poste d’effectuer lui-même la levée de doute incendie</t>
+  </si>
+  <si>
+    <t>[UV11] En cas d’alarme observée sur la centrale incendie, quelle est généralement la procédure à suivre ?</t>
+  </si>
+  <si>
+    <t>Appel de l’astreinte incendie, attente des secours, intervention éventuelle sur le feu</t>
+  </si>
+  <si>
+    <t>Acquittement du signal sonore, lecture de l’information, levée de doute, plan d’action conforme aux consignes du site</t>
+  </si>
+  <si>
+    <t>Levée de doute, appel des secours, retour au PCS</t>
+  </si>
+  <si>
+    <t>Intervention immédiate sur feu, appel des secours, réinitialisation central incendie</t>
+  </si>
+  <si>
+    <t>[UV9] Quelles sont les méthodes pour les agents masculins pour effectuer des vérifications de sécurité sur des femmes qui sont au contrôle d’accès :</t>
+  </si>
+  <si>
+    <t>Le contrôle visuel des bagages</t>
+  </si>
+  <si>
+    <t>[UV9] Dans quelle situation puis-je effectuer des palpations de sécurité ?</t>
+  </si>
+  <si>
+    <t>Dans tout le magasin sur des personnes soupçonnées de vouloir fumer</t>
+  </si>
+  <si>
+    <t>À l’intérieur d’une salle de concert à la demande du chef de poste</t>
+  </si>
+  <si>
+    <t>Dans tout lieu visé par un arrêté préfectoral</t>
+  </si>
+  <si>
+    <t>À la sortie du magasin sur un individu connu pour des actes de vol</t>
+  </si>
+  <si>
+    <t>[UV8] Certaines circonstances peuvent aggraver le vol. Par exemple quand le vol est commis :</t>
+  </si>
+  <si>
+    <t>Par plusieurs personnes</t>
+  </si>
+  <si>
+    <t>Chez une personne dépositaire de l’autorité publique</t>
+  </si>
+  <si>
+    <t>Sur une personne dans la journée</t>
+  </si>
+  <si>
+    <t>Dans un local sous surveillance électronique</t>
+  </si>
+  <si>
+    <t>[UV7] Dès l’arrivée des forces de l’ordre, dans une zone d’attentat, vous devez en premier :</t>
+  </si>
+  <si>
+    <t>Leur parler de la situation</t>
+  </si>
+  <si>
+    <t>Courir vers eux</t>
+  </si>
+  <si>
+    <t>Leur indiquer l’emplacement des victimes</t>
+  </si>
+  <si>
+    <t>Suivre leurs instructions</t>
+  </si>
+  <si>
+    <t>[UV7] Parmi les types de “BLAST” suivants, lequel ou lesquels existent ?</t>
+  </si>
+  <si>
+    <t>BLAST primaire</t>
+  </si>
+  <si>
+    <t>BLAST tertiaire</t>
+  </si>
+  <si>
+    <t>BLAST quaternaire</t>
+  </si>
+  <si>
+    <t>BLAST secondaire</t>
+  </si>
+  <si>
+    <t>[UV2] Agent de sécurité, je dispose d’un véhicule d’entreprise équipé d’un gyrophare orange :</t>
+  </si>
+  <si>
+    <t>C’est absolument interdit</t>
+  </si>
+  <si>
+    <t>C’est autorisé uniquement à l’intérieur des sites surveillés, si les consignes le prévoient</t>
+  </si>
+  <si>
+    <t>Seuls les gyrophares bleus sont autorisés pour les agents de sécurité</t>
+  </si>
+  <si>
+    <t>C’est interdit, sauf en situation d’urgence attentat</t>
+  </si>
+  <si>
+    <t>[UV2] Selon la loi, est une arme par destination :</t>
+  </si>
+  <si>
+    <t>Tout objet conçu pour usage professionnel</t>
+  </si>
+  <si>
+    <t>Tout objet conçu pour tuer ou blesser</t>
+  </si>
+  <si>
+    <t>Tout objet susceptible de présenter un danger pour des personnes, dès lors qu’il est utilisé pour menacer</t>
+  </si>
+  <si>
+    <t>Tout objet pouvant causer des dommages</t>
+  </si>
+  <si>
+    <t>[UV11] Le report d’alarme d’une centrale intrusion est un dispositif :</t>
+  </si>
+  <si>
+    <t>Uniquement destiné aux équipes de sûreté en cas d’intrusion</t>
+  </si>
+  <si>
+    <t>De secours en cas de défaillance du clavier principal</t>
+  </si>
+  <si>
+    <t>Qui permet aux agents d’accéder à certaines informations hors du PCS</t>
+  </si>
+  <si>
+    <t>De cloisonnement anti-intrusion indépendant du système central</t>
+  </si>
+  <si>
+    <t>[UV14] Dans quel document l’APS peut trouver les mesures opératoires des secours extérieurs lors d’un sinistre majeur ?</t>
+  </si>
+  <si>
+    <t>Le Plan des Opérations Externes (P.O.E.)</t>
+  </si>
+  <si>
+    <t>Le Plan Particulier d’Intervention (P.P.I. ou équivalent)</t>
+  </si>
+  <si>
+    <t>Le Plan de Secours Extérieurs (P.S.E.)</t>
+  </si>
+  <si>
+    <t>Le Plan Particulier des Risques Majeurs (P.P.R.M.)</t>
+  </si>
+  <si>
+    <t>[UV14] Quand doit-on rédiger notamment impérativement un Plan de Prévention ?</t>
+  </si>
+  <si>
+    <t>En cas de travaux dangereux listés dans l’arrêté du 19 mars 1993</t>
+  </si>
+  <si>
+    <t>Uniquement lorsque les consignes de sûreté le prévoient</t>
+  </si>
+  <si>
+    <t>Si vous estimez que l’importance des travaux le nécessitent</t>
+  </si>
+  <si>
+    <t>Uniquement sur demande explicite du client</t>
+  </si>
+  <si>
+    <t>[UV14] Quel est l’objectif général de la prévention ?</t>
+  </si>
+  <si>
+    <t>Définir les mesures de sûreté</t>
+  </si>
+  <si>
+    <t>Protéger l’employeur du risque pénal</t>
+  </si>
+  <si>
+    <t>Améliorer les statistiques concernant les taux d’accidents</t>
+  </si>
+  <si>
+    <t>Éviter ou limiter les dommages</t>
+  </si>
+  <si>
+    <t>VRAC 1</t>
+  </si>
+  <si>
+    <t>VRAC 2</t>
+  </si>
+  <si>
+    <t>VRAC 3</t>
+  </si>
+  <si>
+    <t>Questions vrac</t>
+  </si>
+  <si>
+    <t>[UV7] Que signifie le R de NRBC-E ?</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5548,6 +6523,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -5603,7 +6591,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -5648,6 +6636,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6491,10 +7483,10 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:J205"/>
+  <dimension ref="A1:J260"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" style="9" customWidth="1"/>
     <col min="2" max="2" width="9.140625" style="9"/>
     <col min="3" max="3" width="59.28515625" style="2" customWidth="1"/>
     <col min="4" max="9" width="26.7109375" style="2" customWidth="1"/>
@@ -12475,6 +13467,1598 @@
       </c>
       <c r="J205" s="10" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A206" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B206" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C206" s="2" t="s">
+        <v>1506</v>
+      </c>
+      <c r="D206" s="2" t="s">
+        <v>1255</v>
+      </c>
+      <c r="E206" s="2" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F206" s="2" t="s">
+        <v>1257</v>
+      </c>
+      <c r="G206" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H206" s="2" t="s">
+        <v>1258</v>
+      </c>
+      <c r="J206" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A207" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B207" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>1259</v>
+      </c>
+      <c r="D207" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E207" s="2" t="s">
+        <v>1260</v>
+      </c>
+      <c r="F207" s="2" t="s">
+        <v>1261</v>
+      </c>
+      <c r="G207" s="2" t="s">
+        <v>1262</v>
+      </c>
+      <c r="H207" s="2" t="s">
+        <v>1263</v>
+      </c>
+      <c r="J207" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A208" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B208" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C208" s="2" t="s">
+        <v>1264</v>
+      </c>
+      <c r="D208" s="2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="E208" s="2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="F208" s="2" t="s">
+        <v>1267</v>
+      </c>
+      <c r="G208" s="2" t="s">
+        <v>1268</v>
+      </c>
+      <c r="H208" s="2" t="s">
+        <v>1269</v>
+      </c>
+      <c r="J208" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A209" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B209" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C209" s="2" t="s">
+        <v>1270</v>
+      </c>
+      <c r="D209" s="2" t="s">
+        <v>1271</v>
+      </c>
+      <c r="E209" s="2" t="s">
+        <v>1272</v>
+      </c>
+      <c r="F209" s="2" t="s">
+        <v>1273</v>
+      </c>
+      <c r="G209" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H209" s="2" t="s">
+        <v>1274</v>
+      </c>
+      <c r="J209" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A210" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B210" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C210" s="2" t="s">
+        <v>1275</v>
+      </c>
+      <c r="D210" s="2" t="s">
+        <v>1276</v>
+      </c>
+      <c r="E210" s="2" t="s">
+        <v>1277</v>
+      </c>
+      <c r="F210" s="2" t="s">
+        <v>1278</v>
+      </c>
+      <c r="G210" s="2" t="s">
+        <v>1279</v>
+      </c>
+      <c r="H210" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="J210" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A211" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B211" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C211" s="2" t="s">
+        <v>1280</v>
+      </c>
+      <c r="D211" s="2" t="s">
+        <v>1281</v>
+      </c>
+      <c r="E211" s="2" t="s">
+        <v>1282</v>
+      </c>
+      <c r="F211" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="G211" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H211" s="2" t="s">
+        <v>1284</v>
+      </c>
+      <c r="J211" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A212" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B212" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C212" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="D212" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="E212" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="F212" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="G212" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H212" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="J212" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A213" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B213" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C213" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="D213" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="E213" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F213" s="2" t="s">
+        <v>1292</v>
+      </c>
+      <c r="G213" s="2" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H213" s="2" t="s">
+        <v>1294</v>
+      </c>
+      <c r="J213" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A214" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B214" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C214" s="2" t="s">
+        <v>1295</v>
+      </c>
+      <c r="D214" s="2" t="s">
+        <v>1296</v>
+      </c>
+      <c r="E214" s="2" t="s">
+        <v>1297</v>
+      </c>
+      <c r="F214" s="2" t="s">
+        <v>1298</v>
+      </c>
+      <c r="G214" s="2" t="s">
+        <v>1299</v>
+      </c>
+      <c r="H214" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="J214" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A215" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B215" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C215" s="2" t="s">
+        <v>1300</v>
+      </c>
+      <c r="D215" s="2" t="s">
+        <v>1301</v>
+      </c>
+      <c r="E215" s="2" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F215" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G215" s="2" t="s">
+        <v>1303</v>
+      </c>
+      <c r="H215" s="2" t="s">
+        <v>1304</v>
+      </c>
+      <c r="J215" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A216" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B216" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C216" s="2" t="s">
+        <v>1305</v>
+      </c>
+      <c r="D216" s="2" t="s">
+        <v>1306</v>
+      </c>
+      <c r="E216" s="2" t="s">
+        <v>1307</v>
+      </c>
+      <c r="F216" s="2" t="s">
+        <v>1308</v>
+      </c>
+      <c r="G216" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H216" s="2" t="s">
+        <v>1309</v>
+      </c>
+      <c r="J216" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A217" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B217" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C217" s="2" t="s">
+        <v>1310</v>
+      </c>
+      <c r="D217" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E217" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F217" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G217" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H217" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J217" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A218" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B218" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C218" s="2" t="s">
+        <v>1311</v>
+      </c>
+      <c r="D218" s="2" t="s">
+        <v>1312</v>
+      </c>
+      <c r="E218" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F218" s="2" t="s">
+        <v>1313</v>
+      </c>
+      <c r="G218" s="2" t="s">
+        <v>1314</v>
+      </c>
+      <c r="H218" s="2" t="s">
+        <v>1315</v>
+      </c>
+      <c r="J218" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A219" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B219" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>1316</v>
+      </c>
+      <c r="D219" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="E219" s="2" t="s">
+        <v>898</v>
+      </c>
+      <c r="F219" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="G219" s="2" t="s">
+        <v>1317</v>
+      </c>
+      <c r="H219" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J219" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A220" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B220" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>1318</v>
+      </c>
+      <c r="D220" s="2" t="s">
+        <v>1319</v>
+      </c>
+      <c r="E220" s="2" t="s">
+        <v>1320</v>
+      </c>
+      <c r="F220" s="2" t="s">
+        <v>1321</v>
+      </c>
+      <c r="G220" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H220" s="2" t="s">
+        <v>855</v>
+      </c>
+      <c r="J220" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A221" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B221" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C221" s="2" t="s">
+        <v>1322</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>1323</v>
+      </c>
+      <c r="E221" s="2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F221" s="2" t="s">
+        <v>1325</v>
+      </c>
+      <c r="G221" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H221" s="2" t="s">
+        <v>1326</v>
+      </c>
+      <c r="J221" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A222" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B222" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>1327</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E222" s="2" t="s">
+        <v>1328</v>
+      </c>
+      <c r="F222" s="2" t="s">
+        <v>1329</v>
+      </c>
+      <c r="G222" s="2" t="s">
+        <v>1330</v>
+      </c>
+      <c r="H222" s="2" t="s">
+        <v>1331</v>
+      </c>
+      <c r="J222" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A223" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B223" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>1332</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>1333</v>
+      </c>
+      <c r="E223" s="2" t="s">
+        <v>1334</v>
+      </c>
+      <c r="F223" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G223" s="2" t="s">
+        <v>1335</v>
+      </c>
+      <c r="H223" s="2" t="s">
+        <v>1336</v>
+      </c>
+      <c r="J223" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A224" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B224" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>1337</v>
+      </c>
+      <c r="D224" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="E224" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F224" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="G224" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="H224" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="J224" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A225" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B225" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C225" s="2" t="s">
+        <v>1338</v>
+      </c>
+      <c r="D225" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="E225" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F225" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="G225" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="H225" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="J225" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A226" s="9" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B226" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>1339</v>
+      </c>
+      <c r="D226" s="2" t="s">
+        <v>1340</v>
+      </c>
+      <c r="E226" s="2" t="s">
+        <v>1341</v>
+      </c>
+      <c r="F226" s="2" t="s">
+        <v>1342</v>
+      </c>
+      <c r="G226" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H226" s="2" t="s">
+        <v>1343</v>
+      </c>
+      <c r="J226" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A227" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B227" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C227" s="2" t="s">
+        <v>1344</v>
+      </c>
+      <c r="D227" s="2" t="s">
+        <v>1345</v>
+      </c>
+      <c r="E227" s="2" t="s">
+        <v>1346</v>
+      </c>
+      <c r="F227" s="2" t="s">
+        <v>1347</v>
+      </c>
+      <c r="G227" s="2" t="s">
+        <v>1348</v>
+      </c>
+      <c r="H227" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J227" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A228" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B228" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>1349</v>
+      </c>
+      <c r="D228" s="2" t="s">
+        <v>1350</v>
+      </c>
+      <c r="E228" s="2" t="s">
+        <v>1351</v>
+      </c>
+      <c r="F228" s="2" t="s">
+        <v>1352</v>
+      </c>
+      <c r="G228" s="2" t="s">
+        <v>1353</v>
+      </c>
+      <c r="H228" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J228" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A229" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B229" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C229" s="2" t="s">
+        <v>1354</v>
+      </c>
+      <c r="D229" s="2" t="s">
+        <v>1355</v>
+      </c>
+      <c r="E229" s="2" t="s">
+        <v>1356</v>
+      </c>
+      <c r="F229" s="2" t="s">
+        <v>1357</v>
+      </c>
+      <c r="G229" s="2" t="s">
+        <v>1358</v>
+      </c>
+      <c r="H229" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J229" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A230" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B230" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C230" s="2" t="s">
+        <v>1359</v>
+      </c>
+      <c r="D230" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E230" s="2" t="s">
+        <v>1360</v>
+      </c>
+      <c r="F230" s="2" t="s">
+        <v>1361</v>
+      </c>
+      <c r="G230" s="2" t="s">
+        <v>1362</v>
+      </c>
+      <c r="H230" s="2" t="s">
+        <v>1363</v>
+      </c>
+      <c r="J230" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A231" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B231" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C231" s="2" t="s">
+        <v>1364</v>
+      </c>
+      <c r="D231" s="2" t="s">
+        <v>1365</v>
+      </c>
+      <c r="E231" s="2" t="s">
+        <v>1366</v>
+      </c>
+      <c r="F231" s="2" t="s">
+        <v>1367</v>
+      </c>
+      <c r="G231" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J231" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A232" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B232" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C232" s="2" t="s">
+        <v>1368</v>
+      </c>
+      <c r="D232" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E232" s="2" t="s">
+        <v>1369</v>
+      </c>
+      <c r="F232" s="2" t="s">
+        <v>1370</v>
+      </c>
+      <c r="G232" s="2" t="s">
+        <v>1371</v>
+      </c>
+      <c r="H232" s="2" t="s">
+        <v>1372</v>
+      </c>
+      <c r="J232" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A233" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B233" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C233" s="2" t="s">
+        <v>1373</v>
+      </c>
+      <c r="D233" s="2" t="s">
+        <v>1374</v>
+      </c>
+      <c r="E233" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F233" s="2" t="s">
+        <v>1375</v>
+      </c>
+      <c r="G233" s="2" t="s">
+        <v>1376</v>
+      </c>
+      <c r="H233" s="2" t="s">
+        <v>1377</v>
+      </c>
+      <c r="J233" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A234" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B234" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C234" s="2" t="s">
+        <v>1378</v>
+      </c>
+      <c r="D234" s="2" t="s">
+        <v>1379</v>
+      </c>
+      <c r="E234" s="2" t="s">
+        <v>1380</v>
+      </c>
+      <c r="F234" s="2" t="s">
+        <v>1381</v>
+      </c>
+      <c r="G234" s="2" t="s">
+        <v>1382</v>
+      </c>
+      <c r="H234" s="2" t="s">
+        <v>1383</v>
+      </c>
+      <c r="J234" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A235" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B235" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C235" s="2" t="s">
+        <v>1384</v>
+      </c>
+      <c r="D235" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E235" s="2" t="s">
+        <v>1385</v>
+      </c>
+      <c r="F235" s="2" t="s">
+        <v>1386</v>
+      </c>
+      <c r="G235" s="2" t="s">
+        <v>1387</v>
+      </c>
+      <c r="H235" s="2" t="s">
+        <v>1388</v>
+      </c>
+      <c r="J235" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="236" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A236" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B236" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C236" s="2" t="s">
+        <v>1389</v>
+      </c>
+      <c r="D236" s="2" t="s">
+        <v>1390</v>
+      </c>
+      <c r="E236" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F236" s="2" t="s">
+        <v>1391</v>
+      </c>
+      <c r="G236" s="2" t="s">
+        <v>1392</v>
+      </c>
+      <c r="H236" s="2" t="s">
+        <v>1393</v>
+      </c>
+      <c r="J236" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="237" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A237" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B237" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C237" s="2" t="s">
+        <v>1394</v>
+      </c>
+      <c r="D237" s="2" t="s">
+        <v>940</v>
+      </c>
+      <c r="E237" s="2" t="s">
+        <v>1395</v>
+      </c>
+      <c r="F237" s="2" t="s">
+        <v>1396</v>
+      </c>
+      <c r="G237" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H237" s="2" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J237" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="238" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A238" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B238" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C238" s="2" t="s">
+        <v>1398</v>
+      </c>
+      <c r="D238" s="2" t="s">
+        <v>1399</v>
+      </c>
+      <c r="E238" s="2" t="s">
+        <v>1400</v>
+      </c>
+      <c r="F238" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G238" s="2" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H238" s="2" t="s">
+        <v>1401</v>
+      </c>
+      <c r="J238" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="239" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A239" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B239" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C239" s="2" t="s">
+        <v>1402</v>
+      </c>
+      <c r="D239" s="2" t="s">
+        <v>1403</v>
+      </c>
+      <c r="E239" s="2" t="s">
+        <v>1404</v>
+      </c>
+      <c r="F239" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G239" s="2" t="s">
+        <v>1405</v>
+      </c>
+      <c r="H239" s="2" t="s">
+        <v>1406</v>
+      </c>
+      <c r="J239" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="240" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A240" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B240" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C240" s="2" t="s">
+        <v>1407</v>
+      </c>
+      <c r="D240" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="E240" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="F240" s="2" t="s">
+        <v>1408</v>
+      </c>
+      <c r="G240" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H240" s="2" t="s">
+        <v>1409</v>
+      </c>
+      <c r="J240" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="241" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A241" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B241" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C241" s="2" t="s">
+        <v>1410</v>
+      </c>
+      <c r="D241" s="2" t="s">
+        <v>1411</v>
+      </c>
+      <c r="E241" s="2" t="s">
+        <v>1412</v>
+      </c>
+      <c r="F241" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G241" s="2" t="s">
+        <v>1413</v>
+      </c>
+      <c r="H241" s="2" t="s">
+        <v>1414</v>
+      </c>
+      <c r="J241" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="242" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A242" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B242" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C242" s="2" t="s">
+        <v>1415</v>
+      </c>
+      <c r="D242" s="2" t="s">
+        <v>1416</v>
+      </c>
+      <c r="E242" s="2" t="s">
+        <v>1417</v>
+      </c>
+      <c r="F242" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G242" s="2" t="s">
+        <v>1418</v>
+      </c>
+      <c r="H242" s="2" t="s">
+        <v>1419</v>
+      </c>
+      <c r="J242" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="243" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A243" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B243" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C243" s="2" t="s">
+        <v>1420</v>
+      </c>
+      <c r="D243" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E243" s="2" t="s">
+        <v>1421</v>
+      </c>
+      <c r="F243" s="2" t="s">
+        <v>1422</v>
+      </c>
+      <c r="G243" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H243" s="2" t="s">
+        <v>1423</v>
+      </c>
+      <c r="J243" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="244" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A244" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B244" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C244" s="2" t="s">
+        <v>1424</v>
+      </c>
+      <c r="D244" s="2" t="s">
+        <v>881</v>
+      </c>
+      <c r="E244" s="2" t="s">
+        <v>880</v>
+      </c>
+      <c r="F244" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G244" s="2" t="s">
+        <v>883</v>
+      </c>
+      <c r="H244" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="J244" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="245" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A245" s="9" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B245" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C245" s="2" t="s">
+        <v>1425</v>
+      </c>
+      <c r="D245" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E245" s="2" t="s">
+        <v>1426</v>
+      </c>
+      <c r="F245" s="2" t="s">
+        <v>1427</v>
+      </c>
+      <c r="G245" s="2" t="s">
+        <v>1428</v>
+      </c>
+      <c r="H245" s="2" t="s">
+        <v>1429</v>
+      </c>
+      <c r="J245" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="246" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A246" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B246" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C246" s="2" t="s">
+        <v>1430</v>
+      </c>
+      <c r="D246" s="2" t="s">
+        <v>1431</v>
+      </c>
+      <c r="E246" s="2" t="s">
+        <v>1432</v>
+      </c>
+      <c r="F246" s="2" t="s">
+        <v>1433</v>
+      </c>
+      <c r="G246" s="2" t="s">
+        <v>1434</v>
+      </c>
+      <c r="H246" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J246" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="247" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A247" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B247" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C247" s="2" t="s">
+        <v>1435</v>
+      </c>
+      <c r="D247" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E247" s="2" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F247" s="2" t="s">
+        <v>1437</v>
+      </c>
+      <c r="G247" s="2" t="s">
+        <v>1438</v>
+      </c>
+      <c r="H247" s="2" t="s">
+        <v>1439</v>
+      </c>
+      <c r="J247" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="248" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A248" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B248" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C248" s="2" t="s">
+        <v>1440</v>
+      </c>
+      <c r="D248" s="2" t="s">
+        <v>1441</v>
+      </c>
+      <c r="E248" s="2" t="s">
+        <v>1442</v>
+      </c>
+      <c r="F248" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G248" s="2" t="s">
+        <v>1443</v>
+      </c>
+      <c r="H248" s="2" t="s">
+        <v>1444</v>
+      </c>
+      <c r="J248" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="249" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A249" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B249" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C249" s="2" t="s">
+        <v>1445</v>
+      </c>
+      <c r="D249" s="2" t="s">
+        <v>1446</v>
+      </c>
+      <c r="E249" s="2" t="s">
+        <v>1447</v>
+      </c>
+      <c r="F249" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G249" s="2" t="s">
+        <v>1448</v>
+      </c>
+      <c r="H249" s="2" t="s">
+        <v>1449</v>
+      </c>
+      <c r="J249" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="250" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A250" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B250" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C250" s="2" t="s">
+        <v>1450</v>
+      </c>
+      <c r="D250" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="E250" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="F250" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="G250" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H250" s="2" t="s">
+        <v>1451</v>
+      </c>
+      <c r="J250" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="251" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A251" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B251" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C251" s="2" t="s">
+        <v>1452</v>
+      </c>
+      <c r="D251" s="2" t="s">
+        <v>1453</v>
+      </c>
+      <c r="E251" s="2" t="s">
+        <v>1454</v>
+      </c>
+      <c r="F251" s="2" t="s">
+        <v>1455</v>
+      </c>
+      <c r="G251" s="2" t="s">
+        <v>1456</v>
+      </c>
+      <c r="H251" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J251" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="252" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A252" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B252" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C252" s="2" t="s">
+        <v>1457</v>
+      </c>
+      <c r="D252" s="2" t="s">
+        <v>1458</v>
+      </c>
+      <c r="E252" s="2" t="s">
+        <v>1459</v>
+      </c>
+      <c r="F252" s="2" t="s">
+        <v>1460</v>
+      </c>
+      <c r="G252" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H252" s="2" t="s">
+        <v>1461</v>
+      </c>
+      <c r="J252" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="253" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A253" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B253" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C253" s="2" t="s">
+        <v>1462</v>
+      </c>
+      <c r="D253" s="2" t="s">
+        <v>1463</v>
+      </c>
+      <c r="E253" s="2" t="s">
+        <v>1464</v>
+      </c>
+      <c r="F253" s="2" t="s">
+        <v>1465</v>
+      </c>
+      <c r="G253" s="2" t="s">
+        <v>1466</v>
+      </c>
+      <c r="H253" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J253" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="254" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A254" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B254" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C254" s="2" t="s">
+        <v>1467</v>
+      </c>
+      <c r="D254" s="2" t="s">
+        <v>1468</v>
+      </c>
+      <c r="E254" s="2" t="s">
+        <v>1469</v>
+      </c>
+      <c r="F254" s="2" t="s">
+        <v>1470</v>
+      </c>
+      <c r="G254" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="H254" s="2" t="s">
+        <v>1471</v>
+      </c>
+      <c r="J254" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="255" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A255" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B255" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C255" s="2" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D255" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E255" s="2" t="s">
+        <v>1473</v>
+      </c>
+      <c r="F255" s="2" t="s">
+        <v>1474</v>
+      </c>
+      <c r="G255" s="2" t="s">
+        <v>1475</v>
+      </c>
+      <c r="H255" s="2" t="s">
+        <v>1476</v>
+      </c>
+      <c r="J255" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="256" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A256" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B256" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C256" s="2" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D256" s="2" t="s">
+        <v>1478</v>
+      </c>
+      <c r="E256" s="2" t="s">
+        <v>1479</v>
+      </c>
+      <c r="F256" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G256" s="2" t="s">
+        <v>1480</v>
+      </c>
+      <c r="H256" s="2" t="s">
+        <v>1481</v>
+      </c>
+      <c r="J256" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="257" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A257" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B257" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C257" s="2" t="s">
+        <v>1482</v>
+      </c>
+      <c r="D257" s="2" t="s">
+        <v>1483</v>
+      </c>
+      <c r="E257" s="2" t="s">
+        <v>1484</v>
+      </c>
+      <c r="F257" s="2" t="s">
+        <v>1485</v>
+      </c>
+      <c r="G257" s="2" t="s">
+        <v>1486</v>
+      </c>
+      <c r="H257" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J257" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="258" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A258" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B258" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C258" s="2" t="s">
+        <v>1487</v>
+      </c>
+      <c r="D258" s="2" t="s">
+        <v>1488</v>
+      </c>
+      <c r="E258" s="2" t="s">
+        <v>1489</v>
+      </c>
+      <c r="F258" s="2" t="s">
+        <v>1490</v>
+      </c>
+      <c r="G258" s="2" t="s">
+        <v>1491</v>
+      </c>
+      <c r="H258" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J258" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="259" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A259" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B259" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C259" s="2" t="s">
+        <v>1492</v>
+      </c>
+      <c r="D259" s="2" t="s">
+        <v>1493</v>
+      </c>
+      <c r="E259" s="2" t="s">
+        <v>1494</v>
+      </c>
+      <c r="F259" s="2" t="s">
+        <v>1495</v>
+      </c>
+      <c r="G259" s="2" t="s">
+        <v>1496</v>
+      </c>
+      <c r="H259" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J259" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="260" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A260" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B260" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C260" s="2" t="s">
+        <v>1497</v>
+      </c>
+      <c r="D260" s="2" t="s">
+        <v>1498</v>
+      </c>
+      <c r="E260" s="2" t="s">
+        <v>1499</v>
+      </c>
+      <c r="F260" s="2" t="s">
+        <v>1500</v>
+      </c>
+      <c r="G260" s="2" t="s">
+        <v>1501</v>
+      </c>
+      <c r="H260" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J260" s="10" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -12658,18 +15242,42 @@
         <v>269</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="19" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="19" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="19" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13639,13 +16247,14 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18582157-25E0-434E-AB6B-01FE38A60B37}">
-  <dimension ref="A1:I158"/>
+  <dimension ref="A1:J214"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.140625" customWidth="1"/>
@@ -18008,7 +20617,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145" s="6" t="s">
         <v>1011</v>
       </c>
@@ -18040,7 +20649,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146" s="6" t="s">
         <v>1012</v>
       </c>
@@ -18063,7 +20672,7 @@
         <v>Non</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147" s="6" t="s">
         <v>1013</v>
       </c>
@@ -18092,7 +20701,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A148" s="6" t="s">
         <v>1014</v>
       </c>
@@ -18124,7 +20733,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149" s="6" t="s">
         <v>1015</v>
       </c>
@@ -18156,7 +20765,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150" s="6" t="s">
         <v>1016</v>
       </c>
@@ -18188,7 +20797,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151" s="6" t="s">
         <v>1017</v>
       </c>
@@ -18220,7 +20829,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A152" s="6" t="s">
         <v>1018</v>
       </c>
@@ -18252,7 +20861,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153" s="6" t="s">
         <v>1019</v>
       </c>
@@ -18284,7 +20893,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154" s="6" t="s">
         <v>1020</v>
       </c>
@@ -18316,7 +20925,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155" s="6" t="s">
         <v>1021</v>
       </c>
@@ -18348,7 +20957,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156" s="6" t="s">
         <v>1022</v>
       </c>
@@ -18377,7 +20986,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157" s="6" t="s">
         <v>1023</v>
       </c>
@@ -18409,7 +21018,7 @@
         <v>Aucune des réponses précédentes</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158" s="6" t="s">
         <v>1024</v>
       </c>
@@ -18439,6 +21048,1928 @@
       </c>
       <c r="I158" t="str">
         <v>Aucune des réponses précédentes</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A160" s="18" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B160" s="17">
+        <f t="shared" ref="B160" si="20">FIND(" - ",A160)</f>
+        <v>2</v>
+      </c>
+      <c r="C160" s="17" t="str">
+        <f t="shared" ref="C160" si="21">RIGHT(A160, LEN(A160)-(B160+2))</f>
+        <v>[UV7] Que signifie le R de N.R.B.C-E ?|Radiologique|Radicalisé|Radioactif|Aucune des autres réponses|Rayonnant|A</v>
+      </c>
+      <c r="D160" t="str" cm="1">
+        <f t="array" ref="D160:J160">_xlfn.TEXTSPLIT(C160,"|")</f>
+        <v>[UV7] Que signifie le R de N.R.B.C-E ?</v>
+      </c>
+      <c r="E160" t="str">
+        <v>Radiologique</v>
+      </c>
+      <c r="F160" t="str">
+        <v>Radicalisé</v>
+      </c>
+      <c r="G160" t="str">
+        <v>Radioactif</v>
+      </c>
+      <c r="H160" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I160" t="str">
+        <v>Rayonnant</v>
+      </c>
+      <c r="J160" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A161" s="18" t="s">
+        <v>1201</v>
+      </c>
+      <c r="B161" s="17">
+        <f t="shared" ref="B161:B214" si="22">FIND(" - ",A161)</f>
+        <v>2</v>
+      </c>
+      <c r="C161" s="17" t="str">
+        <f t="shared" ref="C161:C214" si="23">RIGHT(A161, LEN(A161)-(B161+2))</f>
+        <v>[UV7] Le Pneumothorax peut être occasionné par :|Toutes les réponses sont bonnes|Une explosion (Blast primaire)|Une perforation par une côte|Une plaie pénétrante par arme blanche|Une plaie pénétrante par balle|A</v>
+      </c>
+      <c r="D161" t="str" cm="1">
+        <f t="array" ref="D161:J161">_xlfn.TEXTSPLIT(C161,"|")</f>
+        <v>[UV7] Le Pneumothorax peut être occasionné par :</v>
+      </c>
+      <c r="E161" t="str">
+        <v>Toutes les réponses sont bonnes</v>
+      </c>
+      <c r="F161" t="str">
+        <v>Une explosion (Blast primaire)</v>
+      </c>
+      <c r="G161" t="str">
+        <v>Une perforation par une côte</v>
+      </c>
+      <c r="H161" t="str">
+        <v>Une plaie pénétrante par arme blanche</v>
+      </c>
+      <c r="I161" t="str">
+        <v>Une plaie pénétrante par balle</v>
+      </c>
+      <c r="J161" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A162" s="18" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B162" s="17">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="C162" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Parmi ces infractions, laquelle porte atteinte aux intérêts fondamentaux de la nation ?|La délation|L’abus de droit public|La rébellion|Le sabotage|La violation de domicile|D</v>
+      </c>
+      <c r="D162" t="str" cm="1">
+        <f t="array" ref="D162:J162">_xlfn.TEXTSPLIT(C162,"|")</f>
+        <v>[UV7] Parmi ces infractions, laquelle porte atteinte aux intérêts fondamentaux de la nation ?</v>
+      </c>
+      <c r="E162" t="str">
+        <v>La délation</v>
+      </c>
+      <c r="F162" t="str">
+        <v>L’abus de droit public</v>
+      </c>
+      <c r="G162" t="str">
+        <v>La rébellion</v>
+      </c>
+      <c r="H162" t="str">
+        <v>Le sabotage</v>
+      </c>
+      <c r="I162" t="str">
+        <v>La violation de domicile</v>
+      </c>
+      <c r="J162" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A163" s="18" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B163" s="17">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="C163" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Dans le cadre d’un risque d’attentat, que peut faire le Préfet ?|Décréter l’état d’urgence, mais seulement au niveau “vigilance”|Faire procéder à des fouilles à corps par des ASP|Accroître les contrôles aux frontières|Aucune des autres réponses|Interdire la circulation, instaurer un couvre-feu et limiter les allées/venues des personnes|E</v>
+      </c>
+      <c r="D163" t="str" cm="1">
+        <f t="array" ref="D163:J163">_xlfn.TEXTSPLIT(C163,"|")</f>
+        <v>[UV7] Dans le cadre d’un risque d’attentat, que peut faire le Préfet ?</v>
+      </c>
+      <c r="E163" t="str">
+        <v>Décréter l’état d’urgence, mais seulement au niveau “vigilance”</v>
+      </c>
+      <c r="F163" t="str">
+        <v>Faire procéder à des fouilles à corps par des ASP</v>
+      </c>
+      <c r="G163" t="str">
+        <v>Accroître les contrôles aux frontières</v>
+      </c>
+      <c r="H163" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I163" t="str">
+        <v>Interdire la circulation, instaurer un couvre-feu et limiter les allées/venues des personnes</v>
+      </c>
+      <c r="J163" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A164" s="18" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B164" s="17">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="C164" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Témoin direct d’un attentat en cours sur votre site, quelles consignes à suivre sont les plus appropriées ?|Alerter les personnes autour de vous|Si possible, aider les autres personnes à s’échapper|Laisser vos affaires derrière vous|Si vous ne pouvez pas courir, se confiner, éteindre la lumière et couper le son des appareils à proximité|Toutes les réponses précédentes sont exactes|E</v>
+      </c>
+      <c r="D164" t="str" cm="1">
+        <f t="array" ref="D164:J164">_xlfn.TEXTSPLIT(C164,"|")</f>
+        <v>[UV7] Témoin direct d’un attentat en cours sur votre site, quelles consignes à suivre sont les plus appropriées ?</v>
+      </c>
+      <c r="E164" t="str">
+        <v>Alerter les personnes autour de vous</v>
+      </c>
+      <c r="F164" t="str">
+        <v>Si possible, aider les autres personnes à s’échapper</v>
+      </c>
+      <c r="G164" t="str">
+        <v>Laisser vos affaires derrière vous</v>
+      </c>
+      <c r="H164" t="str">
+        <v>Si vous ne pouvez pas courir, se confiner, éteindre la lumière et couper le son des appareils à proximité</v>
+      </c>
+      <c r="I164" t="str">
+        <v>Toutes les réponses précédentes sont exactes</v>
+      </c>
+      <c r="J164" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A165" s="18" t="s">
+        <v>1205</v>
+      </c>
+      <c r="B165" s="17">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="C165" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV11] Un groupe d’individus cagoulés et armés pénètre dans votre établissement et vous êtes seul : que faites-vous ?|J’appelle la relève pour me venir en aide le plus tôt possible|Je m’enfuis et je fais appel aux forces de l’ordre le plus rapidement possible|Je m’enfuis si je peux ou sinon je me confine, et je contacte le 114 par sms|Aucune des autres réponses|Je dois agir physiquement pour les expulser de l’établissement|C</v>
+      </c>
+      <c r="D165" t="str" cm="1">
+        <f t="array" ref="D165:J165">_xlfn.TEXTSPLIT(C165,"|")</f>
+        <v>[UV11] Un groupe d’individus cagoulés et armés pénètre dans votre établissement et vous êtes seul : que faites-vous ?</v>
+      </c>
+      <c r="E165" t="str">
+        <v>J’appelle la relève pour me venir en aide le plus tôt possible</v>
+      </c>
+      <c r="F165" t="str">
+        <v>Je m’enfuis et je fais appel aux forces de l’ordre le plus rapidement possible</v>
+      </c>
+      <c r="G165" t="str">
+        <v>Je m’enfuis si je peux ou sinon je me confine, et je contacte le 114 par sms</v>
+      </c>
+      <c r="H165" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I165" t="str">
+        <v>Je dois agir physiquement pour les expulser de l’établissement</v>
+      </c>
+      <c r="J165" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A166" s="18" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B166" s="17">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="C166" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV9] Un agent de prévention et de sécurité a-t-il le droit de pratiquer des palpations de sécurité lors de manifestations sportives, récréatives ou culturelles ?|Oui, en toutes circonstances|Oui, s’il est habilité par son entreprise|Non, sauf s’il est habilité par son employeur|Aucune des autres réponses|Oui, si la manifestation dépasse 300 personnes et sous le contrôle d’un OPJ et que la personne palpée soit du même sexe que l’agent de sécurité|E</v>
+      </c>
+      <c r="D166" t="str" cm="1">
+        <f t="array" ref="D166:J166">_xlfn.TEXTSPLIT(C166,"|")</f>
+        <v>[UV9] Un agent de prévention et de sécurité a-t-il le droit de pratiquer des palpations de sécurité lors de manifestations sportives, récréatives ou culturelles ?</v>
+      </c>
+      <c r="E166" t="str">
+        <v>Oui, en toutes circonstances</v>
+      </c>
+      <c r="F166" t="str">
+        <v>Oui, s’il est habilité par son entreprise</v>
+      </c>
+      <c r="G166" t="str">
+        <v>Non, sauf s’il est habilité par son employeur</v>
+      </c>
+      <c r="H166" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I166" t="str">
+        <v>Oui, si la manifestation dépasse 300 personnes et sous le contrôle d’un OPJ et que la personne palpée soit du même sexe que l’agent de sécurité</v>
+      </c>
+      <c r="J166" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A167" s="18" t="s">
+        <v>1207</v>
+      </c>
+      <c r="B167" s="17">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="C167" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV9] Je suis agent dans un établissement : sous quelles conditions ai-je le droit d’inspecter des sacs ?|Je peux faire une inspection visuelle même si ce n’est pas dans les consignes|Aucune des autres réponses|Si c’est prévu dans les consignes, je peux fouiller les sacs sans avoir besoin du consentement du propriétaire|J’ai le droit de faire une inspection visuelle des bagages et, avec le consentement de leur propriétaire, à leur fouille|Je peux vérifier visuellement et fouiller tous les sacs|D</v>
+      </c>
+      <c r="D167" t="str" cm="1">
+        <f t="array" ref="D167:J167">_xlfn.TEXTSPLIT(C167,"|")</f>
+        <v>[UV9] Je suis agent dans un établissement : sous quelles conditions ai-je le droit d’inspecter des sacs ?</v>
+      </c>
+      <c r="E167" t="str">
+        <v>Je peux faire une inspection visuelle même si ce n’est pas dans les consignes</v>
+      </c>
+      <c r="F167" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="G167" t="str">
+        <v>Si c’est prévu dans les consignes, je peux fouiller les sacs sans avoir besoin du consentement du propriétaire</v>
+      </c>
+      <c r="H167" t="str">
+        <v>J’ai le droit de faire une inspection visuelle des bagages et, avec le consentement de leur propriétaire, à leur fouille</v>
+      </c>
+      <c r="I167" t="str">
+        <v>Je peux vérifier visuellement et fouiller tous les sacs</v>
+      </c>
+      <c r="J167" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A168" s="18" t="s">
+        <v>1208</v>
+      </c>
+      <c r="B168" s="17">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="C168" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV11] En cas de détection incendie, sur quelle unité le voyant est-il lumineux ?|D.A.S.|C.M.S.I.|S.M.S.I.|S.D.I.|Aucune des réponses précédentes|D</v>
+      </c>
+      <c r="D168" t="str" cm="1">
+        <f t="array" ref="D168:J168">_xlfn.TEXTSPLIT(C168,"|")</f>
+        <v>[UV11] En cas de détection incendie, sur quelle unité le voyant est-il lumineux ?</v>
+      </c>
+      <c r="E168" t="str">
+        <v>D.A.S.</v>
+      </c>
+      <c r="F168" t="str">
+        <v>C.M.S.I.</v>
+      </c>
+      <c r="G168" t="str">
+        <v>S.M.S.I.</v>
+      </c>
+      <c r="H168" t="str">
+        <v>S.D.I.</v>
+      </c>
+      <c r="I168" t="str">
+        <v>Aucune des réponses précédentes</v>
+      </c>
+      <c r="J168" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A169" s="18" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B169" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C169" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Que dois-je regarder pour détecter un potentiel terroriste ?|Son comportement|La pratique de sa religion|Aucune des autres réponses|Ses antécédents judiciaires|Son apparence physique|A</v>
+      </c>
+      <c r="D169" t="str" cm="1">
+        <f t="array" ref="D169:J169">_xlfn.TEXTSPLIT(C169,"|")</f>
+        <v>[UV7] Que dois-je regarder pour détecter un potentiel terroriste ?</v>
+      </c>
+      <c r="E169" t="str">
+        <v>Son comportement</v>
+      </c>
+      <c r="F169" t="str">
+        <v>La pratique de sa religion</v>
+      </c>
+      <c r="G169" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H169" t="str">
+        <v>Ses antécédents judiciaires</v>
+      </c>
+      <c r="I169" t="str">
+        <v>Son apparence physique</v>
+      </c>
+      <c r="J169" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A170" s="18" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B170" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C170" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Qu’est-ce que la zone d’exclusion dans un périmètre de sécurité immédiat ?|La zone de prise en charge par les secours|La zone de danger et d’intervention|La zone de commandement des forces de l’ordre|Aucune des autres réponses|La zone d’accueil des force de l’ordre et des secours|B</v>
+      </c>
+      <c r="D170" t="str" cm="1">
+        <f t="array" ref="D170:J170">_xlfn.TEXTSPLIT(C170,"|")</f>
+        <v>[UV7] Qu’est-ce que la zone d’exclusion dans un périmètre de sécurité immédiat ?</v>
+      </c>
+      <c r="E170" t="str">
+        <v>La zone de prise en charge par les secours</v>
+      </c>
+      <c r="F170" t="str">
+        <v>La zone de danger et d’intervention</v>
+      </c>
+      <c r="G170" t="str">
+        <v>La zone de commandement des forces de l’ordre</v>
+      </c>
+      <c r="H170" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I170" t="str">
+        <v>La zone d’accueil des force de l’ordre et des secours</v>
+      </c>
+      <c r="J170" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A171" s="18" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B171" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C171" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV2] Un revolver chambré pour le calibre 38 spécial est une arme de catégorie :|C|D|A|Aucune des autres réponses|B|B</v>
+      </c>
+      <c r="D171" t="str" cm="1">
+        <f t="array" ref="D171:J171">_xlfn.TEXTSPLIT(C171,"|")</f>
+        <v>[UV2] Un revolver chambré pour le calibre 38 spécial est une arme de catégorie :</v>
+      </c>
+      <c r="E171" t="str">
+        <v>C</v>
+      </c>
+      <c r="F171" t="str">
+        <v>D</v>
+      </c>
+      <c r="G171" t="str">
+        <v>A</v>
+      </c>
+      <c r="H171" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I171" t="str">
+        <v>B</v>
+      </c>
+      <c r="J171" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A172" s="18" t="s">
+        <v>1212</v>
+      </c>
+      <c r="B172" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C172" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV2] Le vol avec arme est qualifié de :|Crime terroriste|Aucune des autres réponses|Délit qualifié|Délit aggravé|Crime|E</v>
+      </c>
+      <c r="D172" t="str" cm="1">
+        <f t="array" ref="D172:J172">_xlfn.TEXTSPLIT(C172,"|")</f>
+        <v>[UV2] Le vol avec arme est qualifié de :</v>
+      </c>
+      <c r="E172" t="str">
+        <v>Crime terroriste</v>
+      </c>
+      <c r="F172" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="G172" t="str">
+        <v>Délit qualifié</v>
+      </c>
+      <c r="H172" t="str">
+        <v>Délit aggravé</v>
+      </c>
+      <c r="I172" t="str">
+        <v>Crime</v>
+      </c>
+      <c r="J172" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A173" s="18" t="s">
+        <v>1213</v>
+      </c>
+      <c r="B173" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C173" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] Lorsque des véhicules sont susceptibles de pénétrer au sein de périmètre de protection (L266-1 du CSI), la loi peut également en subordonner l’accès à l’inspection visuelle du contenu du véhicule :|Sans le consentement de son conducteur, par un agent de prévention et de sécurité|Sans le consentement de son conducteur, par un agent de prévention et de sécurité mais sous le contrôle d’un OPJ|Avec le consentement de son conducteur, par un agent de prévention et de sécurité|Avec le consentement de son conducteur, par un agent de prévention et de sécurité placé sous l’autorité d’un OPJ|Aucune des autres réponses|E</v>
+      </c>
+      <c r="D173" t="str" cm="1">
+        <f t="array" ref="D173:J173">_xlfn.TEXTSPLIT(C173,"|")</f>
+        <v>[UV12] Lorsque des véhicules sont susceptibles de pénétrer au sein de périmètre de protection (L266-1 du CSI), la loi peut également en subordonner l’accès à l’inspection visuelle du contenu du véhicule :</v>
+      </c>
+      <c r="E173" t="str">
+        <v>Sans le consentement de son conducteur, par un agent de prévention et de sécurité</v>
+      </c>
+      <c r="F173" t="str">
+        <v>Sans le consentement de son conducteur, par un agent de prévention et de sécurité mais sous le contrôle d’un OPJ</v>
+      </c>
+      <c r="G173" t="str">
+        <v>Avec le consentement de son conducteur, par un agent de prévention et de sécurité</v>
+      </c>
+      <c r="H173" t="str">
+        <v>Avec le consentement de son conducteur, par un agent de prévention et de sécurité placé sous l’autorité d’un OPJ</v>
+      </c>
+      <c r="I173" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J173" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A174" s="18" t="s">
+        <v>1214</v>
+      </c>
+      <c r="B174" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C174" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] Le fait d’accéder frauduleusement à des données informatiques issues d’images de vidéosurveillance constitue l’infraction de :|Atteinte au système de traitement automatisé de données|Entrave à la libre circulation des données|Dégradation ou détérioration d’un système de traitement de données informatiques |Aucune des autres réponses|Vol de données informatiques|A</v>
+      </c>
+      <c r="D174" t="str" cm="1">
+        <f t="array" ref="D174:J174">_xlfn.TEXTSPLIT(C174,"|")</f>
+        <v>[UV12] Le fait d’accéder frauduleusement à des données informatiques issues d’images de vidéosurveillance constitue l’infraction de :</v>
+      </c>
+      <c r="E174" t="str">
+        <v>Atteinte au système de traitement automatisé de données</v>
+      </c>
+      <c r="F174" t="str">
+        <v>Entrave à la libre circulation des données</v>
+      </c>
+      <c r="G174" t="str">
+        <v xml:space="preserve">Dégradation ou détérioration d’un système de traitement de données informatiques </v>
+      </c>
+      <c r="H174" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I174" t="str">
+        <v>Vol de données informatiques</v>
+      </c>
+      <c r="J174" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A175" s="18" t="s">
+        <v>1215</v>
+      </c>
+      <c r="B175" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C175" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] Que signifie l’acronyme P.I.F. dans le cadre d’un système de sécurité lors d’un événement ?|Point ou Poste d’Inspection Filtrage|Poste Itinérant de Filtrage|Passage Interdit à la Foule|Aucune des autres réponses|Permis d’Inspection et de Fouille|A</v>
+      </c>
+      <c r="D175" t="str" cm="1">
+        <f t="array" ref="D175:J175">_xlfn.TEXTSPLIT(C175,"|")</f>
+        <v>[UV12] Que signifie l’acronyme P.I.F. dans le cadre d’un système de sécurité lors d’un événement ?</v>
+      </c>
+      <c r="E175" t="str">
+        <v>Point ou Poste d’Inspection Filtrage</v>
+      </c>
+      <c r="F175" t="str">
+        <v>Poste Itinérant de Filtrage</v>
+      </c>
+      <c r="G175" t="str">
+        <v>Passage Interdit à la Foule</v>
+      </c>
+      <c r="H175" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I175" t="str">
+        <v>Permis d’Inspection et de Fouille</v>
+      </c>
+      <c r="J175" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A176" s="18" t="s">
+        <v>1216</v>
+      </c>
+      <c r="B176" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C176" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] Le plan ORSEC est :|Aucune des autres réponses|Un plan de limitation des déplacements dans le cadre du plan Vigipirates “Urgence Attentat”|Un plan d’Organisation de la Réponses de la Sécurité Civile|Un plan de circulation des riverains lors des événement culturels ou festifs|Un plan d’intervention coordonné des forces de l’ordre publiques et privées|C</v>
+      </c>
+      <c r="D176" t="str" cm="1">
+        <f t="array" ref="D176:J176">_xlfn.TEXTSPLIT(C176,"|")</f>
+        <v>[UV12] Le plan ORSEC est :</v>
+      </c>
+      <c r="E176" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="F176" t="str">
+        <v>Un plan de limitation des déplacements dans le cadre du plan Vigipirates “Urgence Attentat”</v>
+      </c>
+      <c r="G176" t="str">
+        <v>Un plan d’Organisation de la Réponses de la Sécurité Civile</v>
+      </c>
+      <c r="H176" t="str">
+        <v>Un plan de circulation des riverains lors des événement culturels ou festifs</v>
+      </c>
+      <c r="I176" t="str">
+        <v>Un plan d’intervention coordonné des forces de l’ordre publiques et privées</v>
+      </c>
+      <c r="J176" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A177" s="18" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B177" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C177" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV8] Suite à un vol dans un magasin, le chef de poste du PCS reçoit les forces de l’ordre et il peut déposer plainte :|Non, car c’est du ressort exclusif d’un responsable du magasin habilité|Oui, seulement en l’absence du responsable du magasin|Aucune des autres réponses|Oui, car il est le chef de poste et il est donc habilité à déposer plainte|Oui, s’il a l’accord du responsable du magasin|A</v>
+      </c>
+      <c r="D177" t="str" cm="1">
+        <f t="array" ref="D177:J177">_xlfn.TEXTSPLIT(C177,"|")</f>
+        <v>[UV8] Suite à un vol dans un magasin, le chef de poste du PCS reçoit les forces de l’ordre et il peut déposer plainte :</v>
+      </c>
+      <c r="E177" t="str">
+        <v>Non, car c’est du ressort exclusif d’un responsable du magasin habilité</v>
+      </c>
+      <c r="F177" t="str">
+        <v>Oui, seulement en l’absence du responsable du magasin</v>
+      </c>
+      <c r="G177" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H177" t="str">
+        <v>Oui, car il est le chef de poste et il est donc habilité à déposer plainte</v>
+      </c>
+      <c r="I177" t="str">
+        <v>Oui, s’il a l’accord du responsable du magasin</v>
+      </c>
+      <c r="J177" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A178" s="18" t="s">
+        <v>1218</v>
+      </c>
+      <c r="B178" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C178" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV8] Une zone de protection périphérique concerne :|Un objet précis|Aucune des autres réponses|Un local|Une vitrine|Une clôture|E</v>
+      </c>
+      <c r="D178" t="str" cm="1">
+        <f t="array" ref="D178:J178">_xlfn.TEXTSPLIT(C178,"|")</f>
+        <v>[UV8] Une zone de protection périphérique concerne :</v>
+      </c>
+      <c r="E178" t="str">
+        <v>Un objet précis</v>
+      </c>
+      <c r="F178" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="G178" t="str">
+        <v>Un local</v>
+      </c>
+      <c r="H178" t="str">
+        <v>Une vitrine</v>
+      </c>
+      <c r="I178" t="str">
+        <v>Une clôture</v>
+      </c>
+      <c r="J178" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A179" s="18" t="s">
+        <v>1219</v>
+      </c>
+      <c r="B179" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C179" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV8] Une zone de protection ponctuelle concerne :|Un local|Aucune des autres réponses|Une vitrine|Une clôture|Un objet précis|E</v>
+      </c>
+      <c r="D179" t="str" cm="1">
+        <f t="array" ref="D179:J179">_xlfn.TEXTSPLIT(C179,"|")</f>
+        <v>[UV8] Une zone de protection ponctuelle concerne :</v>
+      </c>
+      <c r="E179" t="str">
+        <v>Un local</v>
+      </c>
+      <c r="F179" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="G179" t="str">
+        <v>Une vitrine</v>
+      </c>
+      <c r="H179" t="str">
+        <v>Une clôture</v>
+      </c>
+      <c r="I179" t="str">
+        <v>Un objet précis</v>
+      </c>
+      <c r="J179" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A180" s="18" t="s">
+        <v>1220</v>
+      </c>
+      <c r="B180" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C180" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV8] Les convoyeurs de fonds peuvent-ils être armés lorsqu’ils effectuent en véhicule banalisé un transport de fonds, bijoux ou métaux précieux ?|Oui, avec l’autorisation du Préfet|Non, ils ne peuvent pas être armés|Oui, si la valeur des biens est supérieure à 1,3 millions d’euros|Aucune des autres réponses|Oui sur ordre de la société|B</v>
+      </c>
+      <c r="D180" t="str" cm="1">
+        <f t="array" ref="D180:J180">_xlfn.TEXTSPLIT(C180,"|")</f>
+        <v>[UV8] Les convoyeurs de fonds peuvent-ils être armés lorsqu’ils effectuent en véhicule banalisé un transport de fonds, bijoux ou métaux précieux ?</v>
+      </c>
+      <c r="E180" t="str">
+        <v>Oui, avec l’autorisation du Préfet</v>
+      </c>
+      <c r="F180" t="str">
+        <v>Non, ils ne peuvent pas être armés</v>
+      </c>
+      <c r="G180" t="str">
+        <v>Oui, si la valeur des biens est supérieure à 1,3 millions d’euros</v>
+      </c>
+      <c r="H180" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I180" t="str">
+        <v>Oui sur ordre de la société</v>
+      </c>
+      <c r="J180" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A181" s="18" t="s">
+        <v>1221</v>
+      </c>
+      <c r="B181" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C181" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Que signifie NRBC-E ?|Nationaliste-Radiologique-Bactériologique-Cyberterrorisme et Explosive|Nucléaire-Radiologique-Biologique-Chimique et Explosive|Nucléaire-Radiotechnologique-Bactériologique-Catastrophique et Explosive|Nationaliste-Régionaliste-Bracage-Contrôle et Enlèvement|Aucune des autres réponses|B</v>
+      </c>
+      <c r="D181" t="str" cm="1">
+        <f t="array" ref="D181:J181">_xlfn.TEXTSPLIT(C181,"|")</f>
+        <v>[UV7] Que signifie NRBC-E ?</v>
+      </c>
+      <c r="E181" t="str">
+        <v>Nationaliste-Radiologique-Bactériologique-Cyberterrorisme et Explosive</v>
+      </c>
+      <c r="F181" t="str">
+        <v>Nucléaire-Radiologique-Biologique-Chimique et Explosive</v>
+      </c>
+      <c r="G181" t="str">
+        <v>Nucléaire-Radiotechnologique-Bactériologique-Catastrophique et Explosive</v>
+      </c>
+      <c r="H181" t="str">
+        <v>Nationaliste-Régionaliste-Bracage-Contrôle et Enlèvement</v>
+      </c>
+      <c r="I181" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J181" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A182" s="18" t="s">
+        <v>1222</v>
+      </c>
+      <c r="B182" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C182" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] En cas de plan Vigipirate, l’accès à n’importe quel établissement peut être soumis à une palpation de sécurité : qui peut en décider ?|Le Préfet par un arrêté spécifique|L’agent de sécurité si les consignes spéciales le prévoyants|Le chef d’établissement dans son règlement intérieur|Le CNAPS par une circulaire ministérielle|Aucune des autres réponses|A</v>
+      </c>
+      <c r="D182" t="str" cm="1">
+        <f t="array" ref="D182:J182">_xlfn.TEXTSPLIT(C182,"|")</f>
+        <v>[UV7] En cas de plan Vigipirate, l’accès à n’importe quel établissement peut être soumis à une palpation de sécurité : qui peut en décider ?</v>
+      </c>
+      <c r="E182" t="str">
+        <v>Le Préfet par un arrêté spécifique</v>
+      </c>
+      <c r="F182" t="str">
+        <v>L’agent de sécurité si les consignes spéciales le prévoyants</v>
+      </c>
+      <c r="G182" t="str">
+        <v>Le chef d’établissement dans son règlement intérieur</v>
+      </c>
+      <c r="H182" t="str">
+        <v>Le CNAPS par une circulaire ministérielle</v>
+      </c>
+      <c r="I182" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J182" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A183" s="18" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B183" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C183" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Qu’est-ce que l’état d’urgence ?|Un régime exceptionnel qui permet à l’Etat français de gérer une crise|Un régime qui donne des pouvoirs supplémentaires aux agents de prévention et de sécurité|Un régime continu servant à instaurer un climat de sécurité au peuple|Un régime totalitaire qui octroie les pleins pouvoirs au Président de la République|Aucune des autres réponses|A</v>
+      </c>
+      <c r="D183" t="str" cm="1">
+        <f t="array" ref="D183:J183">_xlfn.TEXTSPLIT(C183,"|")</f>
+        <v>[UV7] Qu’est-ce que l’état d’urgence ?</v>
+      </c>
+      <c r="E183" t="str">
+        <v>Un régime exceptionnel qui permet à l’Etat français de gérer une crise</v>
+      </c>
+      <c r="F183" t="str">
+        <v>Un régime qui donne des pouvoirs supplémentaires aux agents de prévention et de sécurité</v>
+      </c>
+      <c r="G183" t="str">
+        <v>Un régime continu servant à instaurer un climat de sécurité au peuple</v>
+      </c>
+      <c r="H183" t="str">
+        <v>Un régime totalitaire qui octroie les pleins pouvoirs au Président de la République</v>
+      </c>
+      <c r="I183" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J183" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A184" s="18" t="s">
+        <v>1224</v>
+      </c>
+      <c r="B184" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C184" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Suite à une blessure par balle sur le torse d’une victime, comment puis-je la secourir sans provoquer un pneumothorax ?|Aucune des autres réponses|En posant dès que possible un garrot|En réalisant un pansement 3 côtés|En bouchant le trou formé par l’impact avec ma main|En mettant en place la réanimation cardio-pulmonaire|C</v>
+      </c>
+      <c r="D184" t="str" cm="1">
+        <f t="array" ref="D184:J184">_xlfn.TEXTSPLIT(C184,"|")</f>
+        <v>[UV7] Suite à une blessure par balle sur le torse d’une victime, comment puis-je la secourir sans provoquer un pneumothorax ?</v>
+      </c>
+      <c r="E184" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="F184" t="str">
+        <v>En posant dès que possible un garrot</v>
+      </c>
+      <c r="G184" t="str">
+        <v>En réalisant un pansement 3 côtés</v>
+      </c>
+      <c r="H184" t="str">
+        <v>En bouchant le trou formé par l’impact avec ma main</v>
+      </c>
+      <c r="I184" t="str">
+        <v>En mettant en place la réanimation cardio-pulmonaire</v>
+      </c>
+      <c r="J184" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A185" s="18" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B185" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C185" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Quelles sont les grandes priorités de réaction que je dois adopter face à une attaque terroriste ?|Courir, m'enfermer, appeler, attaquer si nécessaire|M’échapper, me cacher, secourir, combattre systématiquement|Alerter, éteindre, méloigner, boxer|Aucune des autres réponses|A</v>
+      </c>
+      <c r="D185" t="str" cm="1">
+        <f t="array" ref="D185:I185">_xlfn.TEXTSPLIT(C185,"|")</f>
+        <v>[UV7] Quelles sont les grandes priorités de réaction que je dois adopter face à une attaque terroriste ?</v>
+      </c>
+      <c r="E185" t="str">
+        <v>Courir, m'enfermer, appeler, attaquer si nécessaire</v>
+      </c>
+      <c r="F185" t="str">
+        <v>M’échapper, me cacher, secourir, combattre systématiquement</v>
+      </c>
+      <c r="G185" t="str">
+        <v>Alerter, éteindre, méloigner, boxer</v>
+      </c>
+      <c r="H185" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I185" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A186" s="18" t="s">
+        <v>1226</v>
+      </c>
+      <c r="B186" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C186" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Qu’est-ce que le terrorisme d’Etat ?|Aucune des autres réponses|Lorsqu’un peuple terrorise son gouvernement|Lorsqu’un Etat terrorise son peuple|Lorsqu’un Etat combat de le terrorisme à l’intérieur de ses frontières|Lorsqu’une organisation terroriste veut prendre le pouvoir d’un Etat|C</v>
+      </c>
+      <c r="D186" t="str" cm="1">
+        <f t="array" ref="D186:J186">_xlfn.TEXTSPLIT(C186,"|")</f>
+        <v>[UV7] Qu’est-ce que le terrorisme d’Etat ?</v>
+      </c>
+      <c r="E186" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="F186" t="str">
+        <v>Lorsqu’un peuple terrorise son gouvernement</v>
+      </c>
+      <c r="G186" t="str">
+        <v>Lorsqu’un Etat terrorise son peuple</v>
+      </c>
+      <c r="H186" t="str">
+        <v>Lorsqu’un Etat combat de le terrorisme à l’intérieur de ses frontières</v>
+      </c>
+      <c r="I186" t="str">
+        <v>Lorsqu’une organisation terroriste veut prendre le pouvoir d’un Etat</v>
+      </c>
+      <c r="J186" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A187" s="18" t="s">
+        <v>1227</v>
+      </c>
+      <c r="B187" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C187" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV2] Un agent de sécurité exerçant ses fonctions dans un parc d’attraction peut-il appréhender un individu qui y entre avec une matraque et tente d’agresser un salarié du parc ?|Il peut juste l’aborder mais il ne peut pas l’appréhender en vertu de l’art. 73 du CPP|Aucune des autres réponses|Oui, car il sera dans le cadre de l’état de nécessité prévu dans l’art. 121-2 du Code Pénal|Non, car il n’y a pas d’infraction prévue pour ce type de fait|Le port d’une matraque constituant un délit, il peut appréhender l’individu au titre de l’art. 73 du CPP|E</v>
+      </c>
+      <c r="D187" t="str" cm="1">
+        <f t="array" ref="D187:J187">_xlfn.TEXTSPLIT(C187,"|")</f>
+        <v>[UV2] Un agent de sécurité exerçant ses fonctions dans un parc d’attraction peut-il appréhender un individu qui y entre avec une matraque et tente d’agresser un salarié du parc ?</v>
+      </c>
+      <c r="E187" t="str">
+        <v>Il peut juste l’aborder mais il ne peut pas l’appréhender en vertu de l’art. 73 du CPP</v>
+      </c>
+      <c r="F187" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="G187" t="str">
+        <v>Oui, car il sera dans le cadre de l’état de nécessité prévu dans l’art. 121-2 du Code Pénal</v>
+      </c>
+      <c r="H187" t="str">
+        <v>Non, car il n’y a pas d’infraction prévue pour ce type de fait</v>
+      </c>
+      <c r="I187" t="str">
+        <v>Le port d’une matraque constituant un délit, il peut appréhender l’individu au titre de l’art. 73 du CPP</v>
+      </c>
+      <c r="J187" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A188" s="18" t="s">
+        <v>1228</v>
+      </c>
+      <c r="B188" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C188" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV2] Un agent de sécurité privé peut être sanctionné par le CNAPS :|À une pénalité financière mais sans limite prise en charge par l’entreprise|À aucune pénalité financière|À une pénalité financière allant jusqu’à 10 000 euros|À une pénalité financière allant jusqu’à 7 500 euros|À une pénalité financière inférieure à 1 500 euros|D</v>
+      </c>
+      <c r="D188" t="str" cm="1">
+        <f t="array" ref="D188:J188">_xlfn.TEXTSPLIT(C188,"|")</f>
+        <v>[UV2] Un agent de sécurité privé peut être sanctionné par le CNAPS :</v>
+      </c>
+      <c r="E188" t="str">
+        <v>À une pénalité financière mais sans limite prise en charge par l’entreprise</v>
+      </c>
+      <c r="F188" t="str">
+        <v>À aucune pénalité financière</v>
+      </c>
+      <c r="G188" t="str">
+        <v>À une pénalité financière allant jusqu’à 10 000 euros</v>
+      </c>
+      <c r="H188" t="str">
+        <v>À une pénalité financière allant jusqu’à 7 500 euros</v>
+      </c>
+      <c r="I188" t="str">
+        <v>À une pénalité financière inférieure à 1 500 euros</v>
+      </c>
+      <c r="J188" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A189" s="18" t="s">
+        <v>1229</v>
+      </c>
+      <c r="B189" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C189" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] À quoi peut servir un PPI/POI/PER ?|Aucune des autres réponses|À coordonner les moyens internes des installations classées|À prévoir la mobilisation des services de secours publics|À protéger les installations recevant du public|À planifier les opérations de maintien de l’ordre|C</v>
+      </c>
+      <c r="D189" t="str" cm="1">
+        <f t="array" ref="D189:J189">_xlfn.TEXTSPLIT(C189,"|")</f>
+        <v>[UV12] À quoi peut servir un PPI/POI/PER ?</v>
+      </c>
+      <c r="E189" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="F189" t="str">
+        <v>À coordonner les moyens internes des installations classées</v>
+      </c>
+      <c r="G189" t="str">
+        <v>À prévoir la mobilisation des services de secours publics</v>
+      </c>
+      <c r="H189" t="str">
+        <v>À protéger les installations recevant du public</v>
+      </c>
+      <c r="I189" t="str">
+        <v>À planifier les opérations de maintien de l’ordre</v>
+      </c>
+      <c r="J189" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A190" s="18" t="s">
+        <v>1230</v>
+      </c>
+      <c r="B190" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C190" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] Il est puni par le code du sport (L332-3) dans une enceinte sportive, lors du déroulement ou de la retransmission en public d’une manifestation sportive :|Le fait d’introduire ou de tenter d’introduire, par force ou par fraude, des boissons alcoolisées|Toutes les réponses sont exactes|Le fait d’avoir, en état d’ivresse, pénétré ou tenté de pénétrer par force ou par fraude|D’un an d’emprisonnement ou d’amende|Le fait d’accéder en état d’ivresse|A</v>
+      </c>
+      <c r="D190" t="str" cm="1">
+        <f t="array" ref="D190:J190">_xlfn.TEXTSPLIT(C190,"|")</f>
+        <v>[UV12] Il est puni par le code du sport (L332-3) dans une enceinte sportive, lors du déroulement ou de la retransmission en public d’une manifestation sportive :</v>
+      </c>
+      <c r="E190" t="str">
+        <v>Le fait d’introduire ou de tenter d’introduire, par force ou par fraude, des boissons alcoolisées</v>
+      </c>
+      <c r="F190" t="str">
+        <v>Toutes les réponses sont exactes</v>
+      </c>
+      <c r="G190" t="str">
+        <v>Le fait d’avoir, en état d’ivresse, pénétré ou tenté de pénétrer par force ou par fraude</v>
+      </c>
+      <c r="H190" t="str">
+        <v>D’un an d’emprisonnement ou d’amende</v>
+      </c>
+      <c r="I190" t="str">
+        <v>Le fait d’accéder en état d’ivresse</v>
+      </c>
+      <c r="J190" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A191" s="18" t="s">
+        <v>1231</v>
+      </c>
+      <c r="B191" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C191" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] Les organisateurs de manifestations sportives, récréatives ou culturelles sont tenus (R211-22 du CSI) :|D’en faire la déclaration uniquement si elles sont sur la liste des événements exposés|D’en faire la déclaration au Préfet de région au moins un an avant l’événement|D’en faire la déclaration aux maires ou aux Préfets de police, si la manifestation peut atteindre plus de 1500 personnes|Aucune des autres réponses|D’en faire la déclaration aux maires si la manifestation peut atteindre plus de 300 personnes et aux Préfets si elle dépasse plus de 1500 personnes|C</v>
+      </c>
+      <c r="D191" t="str" cm="1">
+        <f t="array" ref="D191:J191">_xlfn.TEXTSPLIT(C191,"|")</f>
+        <v>[UV12] Les organisateurs de manifestations sportives, récréatives ou culturelles sont tenus (R211-22 du CSI) :</v>
+      </c>
+      <c r="E191" t="str">
+        <v>D’en faire la déclaration uniquement si elles sont sur la liste des événements exposés</v>
+      </c>
+      <c r="F191" t="str">
+        <v>D’en faire la déclaration au Préfet de région au moins un an avant l’événement</v>
+      </c>
+      <c r="G191" t="str">
+        <v>D’en faire la déclaration aux maires ou aux Préfets de police, si la manifestation peut atteindre plus de 1500 personnes</v>
+      </c>
+      <c r="H191" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I191" t="str">
+        <v>D’en faire la déclaration aux maires si la manifestation peut atteindre plus de 300 personnes et aux Préfets si elle dépasse plus de 1500 personnes</v>
+      </c>
+      <c r="J191" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A192" s="18" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B192" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C192" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV9] Je suis agent dans un magasin : sous quelles conditions ai-je le droit d’inspecter des sacs ?|Je peux faire une inspection visuelle, dès lors que j’ai un doute|Je peux vérifier visuellement et fouiller les sacs sans avoir besoin du consentement du propriétaire|Aucune des autres réponses|J’ai le droit de faire une inspection visuelle des bagages et, avec le consentement de leur propriétaire, à leur fouille|Si c’est prévu dans les consignes, je peux vérifier visuellement et fouiller les sacs sans avoir besoin du consentement du propriétaires|D</v>
+      </c>
+      <c r="D192" t="str" cm="1">
+        <f t="array" ref="D192:J192">_xlfn.TEXTSPLIT(C192,"|")</f>
+        <v>[UV9] Je suis agent dans un magasin : sous quelles conditions ai-je le droit d’inspecter des sacs ?</v>
+      </c>
+      <c r="E192" t="str">
+        <v>Je peux faire une inspection visuelle, dès lors que j’ai un doute</v>
+      </c>
+      <c r="F192" t="str">
+        <v>Je peux vérifier visuellement et fouiller les sacs sans avoir besoin du consentement du propriétaire</v>
+      </c>
+      <c r="G192" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H192" t="str">
+        <v>J’ai le droit de faire une inspection visuelle des bagages et, avec le consentement de leur propriétaire, à leur fouille</v>
+      </c>
+      <c r="I192" t="str">
+        <v>Si c’est prévu dans les consignes, je peux vérifier visuellement et fouiller les sacs sans avoir besoin du consentement du propriétaires</v>
+      </c>
+      <c r="J192" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A193" s="18" t="s">
+        <v>1233</v>
+      </c>
+      <c r="B193" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C193" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV8] Qu’est-ce qu’une zone de protection ?|Lieu protégé par des filets empêchant l’introduction de pigeons dans le site|Lieu protégé par des paroies possédant une isolation phonique|Aucune des autres réponses|Lieu protégé contre les intempéries|Lieu protégé par un obstacle s’opposant à pénétration d’intrus dans le site|E</v>
+      </c>
+      <c r="D193" t="str" cm="1">
+        <f t="array" ref="D193:J193">_xlfn.TEXTSPLIT(C193,"|")</f>
+        <v>[UV8] Qu’est-ce qu’une zone de protection ?</v>
+      </c>
+      <c r="E193" t="str">
+        <v>Lieu protégé par des filets empêchant l’introduction de pigeons dans le site</v>
+      </c>
+      <c r="F193" t="str">
+        <v>Lieu protégé par des paroies possédant une isolation phonique</v>
+      </c>
+      <c r="G193" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H193" t="str">
+        <v>Lieu protégé contre les intempéries</v>
+      </c>
+      <c r="I193" t="str">
+        <v>Lieu protégé par un obstacle s’opposant à pénétration d’intrus dans le site</v>
+      </c>
+      <c r="J193" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A194" s="18" t="s">
+        <v>1234</v>
+      </c>
+      <c r="B194" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C194" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV8] Un point dit vulnérable lors d’une ronde est :|Un point comportant un danger permanent|Un point qui en cas d’atteinte pourrait handicaper le bon fonctionnement de l’entreprise|Un point régulièrement mis en défaut|Aucune des autres réponses|Un point sensible convoité par les voleurs|B</v>
+      </c>
+      <c r="D194" t="str" cm="1">
+        <f t="array" ref="D194:J194">_xlfn.TEXTSPLIT(C194,"|")</f>
+        <v>[UV8] Un point dit vulnérable lors d’une ronde est :</v>
+      </c>
+      <c r="E194" t="str">
+        <v>Un point comportant un danger permanent</v>
+      </c>
+      <c r="F194" t="str">
+        <v>Un point qui en cas d’atteinte pourrait handicaper le bon fonctionnement de l’entreprise</v>
+      </c>
+      <c r="G194" t="str">
+        <v>Un point régulièrement mis en défaut</v>
+      </c>
+      <c r="H194" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I194" t="str">
+        <v>Un point sensible convoité par les voleurs</v>
+      </c>
+      <c r="J194" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A195" s="18" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B195" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C195" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV8] Pendant votre ronde, vous découvrez un local en désordre avec un pied de biche au sol. Que faites-vous ?|Vous ramassez le pied de biche afin d’avoir un objet pour vous défendre|Vous prévenez immédiatement le PCS et inspecter prudemment les locaux voisins|Aucune des autres réponses|Vous ne faites rien et continuez votre rondre, c’est sûrement le bureau d’un salarié désordonné|Vous refermez la porte et prévenez le PCS|B</v>
+      </c>
+      <c r="D195" t="str" cm="1">
+        <f t="array" ref="D195:J195">_xlfn.TEXTSPLIT(C195,"|")</f>
+        <v>[UV8] Pendant votre ronde, vous découvrez un local en désordre avec un pied de biche au sol. Que faites-vous ?</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Vous ramassez le pied de biche afin d’avoir un objet pour vous défendre</v>
+      </c>
+      <c r="F195" t="str">
+        <v>Vous prévenez immédiatement le PCS et inspecter prudemment les locaux voisins</v>
+      </c>
+      <c r="G195" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H195" t="str">
+        <v>Vous ne faites rien et continuez votre rondre, c’est sûrement le bureau d’un salarié désordonné</v>
+      </c>
+      <c r="I195" t="str">
+        <v>Vous refermez la porte et prévenez le PCS</v>
+      </c>
+      <c r="J195" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A196" s="18" t="s">
+        <v>1236</v>
+      </c>
+      <c r="B196" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C196" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV6] Un agent de sécurité privé masculin doit appréhender un voleur en sortie de caisse, mais il s’agit d’une femme :|Il doit appeler une collègue du même sexe|Il agit normalement, néanmoins il est conseillé d’appeler un témoin féminin|Aucune des autres réponses|Il doit demander l’autorisation de la personne|Il ne peut rien faire sur une personne de sexe opposé|B</v>
+      </c>
+      <c r="D196" t="str" cm="1">
+        <f t="array" ref="D196:J196">_xlfn.TEXTSPLIT(C196,"|")</f>
+        <v>[UV6] Un agent de sécurité privé masculin doit appréhender un voleur en sortie de caisse, mais il s’agit d’une femme :</v>
+      </c>
+      <c r="E196" t="str">
+        <v>Il doit appeler une collègue du même sexe</v>
+      </c>
+      <c r="F196" t="str">
+        <v>Il agit normalement, néanmoins il est conseillé d’appeler un témoin féminin</v>
+      </c>
+      <c r="G196" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H196" t="str">
+        <v>Il doit demander l’autorisation de la personne</v>
+      </c>
+      <c r="I196" t="str">
+        <v>Il ne peut rien faire sur une personne de sexe opposé</v>
+      </c>
+      <c r="J196" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A197" s="18" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B197" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C197" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV2] Les agents de sécurité employés par un bailleur d’immeuble à usage d’habitations peuvent être armés :|D’un bâton de défense de type TONFA|D’un fusil à pompe|D’une grenade lacrymogène ayant une capacité inférieure à 100 ml|Aucune des autres réponses|D’un pistolet mitrailleur|A</v>
+      </c>
+      <c r="D197" t="str" cm="1">
+        <f t="array" ref="D197:J197">_xlfn.TEXTSPLIT(C197,"|")</f>
+        <v>[UV2] Les agents de sécurité employés par un bailleur d’immeuble à usage d’habitations peuvent être armés :</v>
+      </c>
+      <c r="E197" t="str">
+        <v>D’un bâton de défense de type TONFA</v>
+      </c>
+      <c r="F197" t="str">
+        <v>D’un fusil à pompe</v>
+      </c>
+      <c r="G197" t="str">
+        <v>D’une grenade lacrymogène ayant une capacité inférieure à 100 ml</v>
+      </c>
+      <c r="H197" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I197" t="str">
+        <v>D’un pistolet mitrailleur</v>
+      </c>
+      <c r="J197" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A198" s="18" t="s">
+        <v>1238</v>
+      </c>
+      <c r="B198" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C198" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] Le schéma d’installation de la vidéoprotection permet :|D’installer, de maintenir et de mettre à disposition des prestataires des images|De capter, de transmettre, de stocker, de visionner les images|Aucune des autres réponses|De garantir aux forces de l’ordre la bonne réalisation de la mission de sûreté|De compléter le système de surveillance incendie|B</v>
+      </c>
+      <c r="D198" t="str" cm="1">
+        <f t="array" ref="D198:J198">_xlfn.TEXTSPLIT(C198,"|")</f>
+        <v>[UV12] Le schéma d’installation de la vidéoprotection permet :</v>
+      </c>
+      <c r="E198" t="str">
+        <v>D’installer, de maintenir et de mettre à disposition des prestataires des images</v>
+      </c>
+      <c r="F198" t="str">
+        <v>De capter, de transmettre, de stocker, de visionner les images</v>
+      </c>
+      <c r="G198" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H198" t="str">
+        <v>De garantir aux forces de l’ordre la bonne réalisation de la mission de sûreté</v>
+      </c>
+      <c r="I198" t="str">
+        <v>De compléter le système de surveillance incendie</v>
+      </c>
+      <c r="J198" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A199" s="18" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B199" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C199" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] À quoi correspond une crash barrière ?|Aucune des autres réponses|Un système de barrière type passage à niveau pour bloquer les accès|Des barrières de sécurité équipés de pieds empêchant le renversement|Un test en laboratoire de la résistance des barrières|L’action de lancer des barrières sur des véhicules voulant forcer l’accès|C</v>
+      </c>
+      <c r="D199" t="str" cm="1">
+        <f t="array" ref="D199:J199">_xlfn.TEXTSPLIT(C199,"|")</f>
+        <v>[UV12] À quoi correspond une crash barrière ?</v>
+      </c>
+      <c r="E199" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="F199" t="str">
+        <v>Un système de barrière type passage à niveau pour bloquer les accès</v>
+      </c>
+      <c r="G199" t="str">
+        <v>Des barrières de sécurité équipés de pieds empêchant le renversement</v>
+      </c>
+      <c r="H199" t="str">
+        <v>Un test en laboratoire de la résistance des barrières</v>
+      </c>
+      <c r="I199" t="str">
+        <v>L’action de lancer des barrières sur des véhicules voulant forcer l’accès</v>
+      </c>
+      <c r="J199" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A200" s="18" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B200" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C200" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV12] Un APS effectue une ronde dans la chaufferie gaz, il peut y entrer si :|Il dispose d’une radio fabriquée après le 1er juillet 2017|Il dispose d’un matériel anti-déflagrant|Il dispose d’un émetteur multi-fréquences|Il dispose d’une pastille de détection de gaz homologuée|Aucune des autres réponses|B</v>
+      </c>
+      <c r="D200" t="str" cm="1">
+        <f t="array" ref="D200:J200">_xlfn.TEXTSPLIT(C200,"|")</f>
+        <v>[UV12] Un APS effectue une ronde dans la chaufferie gaz, il peut y entrer si :</v>
+      </c>
+      <c r="E200" t="str">
+        <v>Il dispose d’une radio fabriquée après le 1er juillet 2017</v>
+      </c>
+      <c r="F200" t="str">
+        <v>Il dispose d’un matériel anti-déflagrant</v>
+      </c>
+      <c r="G200" t="str">
+        <v>Il dispose d’un émetteur multi-fréquences</v>
+      </c>
+      <c r="H200" t="str">
+        <v>Il dispose d’une pastille de détection de gaz homologuée</v>
+      </c>
+      <c r="I200" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J200" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A201" s="18" t="s">
+        <v>1241</v>
+      </c>
+      <c r="B201" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C201" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV11] Sur votre GTB/GTC vous recevez une alarme SURCHAUFF au niveau de la chaufferie. Que devez-vous faire en premier ?|Aucune des autres réponses|Arrêter le signal sonore de l’alarme|Appeler les services de secours|Couper la chaudière|Appeler le technicien compétent|B</v>
+      </c>
+      <c r="D201" t="str" cm="1">
+        <f t="array" ref="D201:J201">_xlfn.TEXTSPLIT(C201,"|")</f>
+        <v>[UV11] Sur votre GTB/GTC vous recevez une alarme SURCHAUFF au niveau de la chaufferie. Que devez-vous faire en premier ?</v>
+      </c>
+      <c r="E201" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="F201" t="str">
+        <v>Arrêter le signal sonore de l’alarme</v>
+      </c>
+      <c r="G201" t="str">
+        <v>Appeler les services de secours</v>
+      </c>
+      <c r="H201" t="str">
+        <v>Couper la chaudière</v>
+      </c>
+      <c r="I201" t="str">
+        <v>Appeler le technicien compétent</v>
+      </c>
+      <c r="J201" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A202" s="18" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B202" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C202" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV11] En vous rendant sur une levée de doute intrusion, votre PC vous appelle car une détection incendie vient d’avoir lieu. Que faites-vous ?|Je termine la levée de doute intrusion sans effectuer les contrôles de rigueur pour aller sur la levée de doute incendie|Je fais demi-tour et priorise la détection incendie dont la gravité peut être supérieure|Aucune des autres réponses|Je poursuis la levée de doute intrusion, étant presque arrivé|Je demande au chef de poste d’effectuer lui-même la levée de doute incendie|B</v>
+      </c>
+      <c r="D202" t="str" cm="1">
+        <f t="array" ref="D202:J202">_xlfn.TEXTSPLIT(C202,"|")</f>
+        <v>[UV11] En vous rendant sur une levée de doute intrusion, votre PC vous appelle car une détection incendie vient d’avoir lieu. Que faites-vous ?</v>
+      </c>
+      <c r="E202" t="str">
+        <v>Je termine la levée de doute intrusion sans effectuer les contrôles de rigueur pour aller sur la levée de doute incendie</v>
+      </c>
+      <c r="F202" t="str">
+        <v>Je fais demi-tour et priorise la détection incendie dont la gravité peut être supérieure</v>
+      </c>
+      <c r="G202" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H202" t="str">
+        <v>Je poursuis la levée de doute intrusion, étant presque arrivé</v>
+      </c>
+      <c r="I202" t="str">
+        <v>Je demande au chef de poste d’effectuer lui-même la levée de doute incendie</v>
+      </c>
+      <c r="J202" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A203" s="18" t="s">
+        <v>1243</v>
+      </c>
+      <c r="B203" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C203" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV11] En cas d’alarme observée sur la centrale incendie, quelle est généralement la procédure à suivre ?|Appel de l’astreinte incendie, attente des secours, intervention éventuelle sur le feu|Acquittement du signal sonore, lecture de l’information, levée de doute, plan d’action conforme aux consignes du site|Aucune des autres réponses|Levée de doute, appel des secours, retour au PCS|Intervention immédiate sur feu, appel des secours, réinitialisation central incendie|B</v>
+      </c>
+      <c r="D203" t="str" cm="1">
+        <f t="array" ref="D203:J203">_xlfn.TEXTSPLIT(C203,"|")</f>
+        <v>[UV11] En cas d’alarme observée sur la centrale incendie, quelle est généralement la procédure à suivre ?</v>
+      </c>
+      <c r="E203" t="str">
+        <v>Appel de l’astreinte incendie, attente des secours, intervention éventuelle sur le feu</v>
+      </c>
+      <c r="F203" t="str">
+        <v>Acquittement du signal sonore, lecture de l’information, levée de doute, plan d’action conforme aux consignes du site</v>
+      </c>
+      <c r="G203" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H203" t="str">
+        <v>Levée de doute, appel des secours, retour au PCS</v>
+      </c>
+      <c r="I203" t="str">
+        <v>Intervention immédiate sur feu, appel des secours, réinitialisation central incendie</v>
+      </c>
+      <c r="J203" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A204" s="18" t="s">
+        <v>1244</v>
+      </c>
+      <c r="B204" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C204" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV9] Quelles sont les méthodes pour les agents masculins pour effectuer des vérifications de sécurité sur des femmes qui sont au contrôle d’accès :|Les palpations de sécurité|La fouille à corps uniquement avec le consentement de la personne|La fouille au corps|Aucune des autres réponses|Le contrôle visuel des bagages|E</v>
+      </c>
+      <c r="D204" t="str" cm="1">
+        <f t="array" ref="D204:J204">_xlfn.TEXTSPLIT(C204,"|")</f>
+        <v>[UV9] Quelles sont les méthodes pour les agents masculins pour effectuer des vérifications de sécurité sur des femmes qui sont au contrôle d’accès :</v>
+      </c>
+      <c r="E204" t="str">
+        <v>Les palpations de sécurité</v>
+      </c>
+      <c r="F204" t="str">
+        <v>La fouille à corps uniquement avec le consentement de la personne</v>
+      </c>
+      <c r="G204" t="str">
+        <v>La fouille au corps</v>
+      </c>
+      <c r="H204" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I204" t="str">
+        <v>Le contrôle visuel des bagages</v>
+      </c>
+      <c r="J204" t="str">
+        <v>E</v>
+      </c>
+    </row>
+    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A205" s="18" t="s">
+        <v>1245</v>
+      </c>
+      <c r="B205" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C205" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV9] Dans quelle situation puis-je effectuer des palpations de sécurité ?|Dans tout le magasin sur des personnes soupçonnées de vouloir fumer|À l’intérieur d’une salle de concert à la demande du chef de poste|Dans tout lieu visé par un arrêté préfectoral|À la sortie du magasin sur un individu connu pour des actes de vol|Aucune des autres réponses|C</v>
+      </c>
+      <c r="D205" t="str" cm="1">
+        <f t="array" ref="D205:J205">_xlfn.TEXTSPLIT(C205,"|")</f>
+        <v>[UV9] Dans quelle situation puis-je effectuer des palpations de sécurité ?</v>
+      </c>
+      <c r="E205" t="str">
+        <v>Dans tout le magasin sur des personnes soupçonnées de vouloir fumer</v>
+      </c>
+      <c r="F205" t="str">
+        <v>À l’intérieur d’une salle de concert à la demande du chef de poste</v>
+      </c>
+      <c r="G205" t="str">
+        <v>Dans tout lieu visé par un arrêté préfectoral</v>
+      </c>
+      <c r="H205" t="str">
+        <v>À la sortie du magasin sur un individu connu pour des actes de vol</v>
+      </c>
+      <c r="I205" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J205" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A206" s="18" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B206" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C206" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV8] Certaines circonstances peuvent aggraver le vol. Par exemple quand le vol est commis :|Par plusieurs personnes|Chez une personne dépositaire de l’autorité publique|Sur une personne dans la journée|Aucune des autres réponses|Dans un local sous surveillance électronique|A</v>
+      </c>
+      <c r="D206" t="str" cm="1">
+        <f t="array" ref="D206:J206">_xlfn.TEXTSPLIT(C206,"|")</f>
+        <v>[UV8] Certaines circonstances peuvent aggraver le vol. Par exemple quand le vol est commis :</v>
+      </c>
+      <c r="E206" t="str">
+        <v>Par plusieurs personnes</v>
+      </c>
+      <c r="F206" t="str">
+        <v>Chez une personne dépositaire de l’autorité publique</v>
+      </c>
+      <c r="G206" t="str">
+        <v>Sur une personne dans la journée</v>
+      </c>
+      <c r="H206" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="I206" t="str">
+        <v>Dans un local sous surveillance électronique</v>
+      </c>
+      <c r="J206" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A207" s="18" t="s">
+        <v>1247</v>
+      </c>
+      <c r="B207" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C207" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Dès l’arrivée des forces de l’ordre, dans une zone d’attentat, vous devez en premier :|Leur parler de la situation|Courir vers eux|Leur indiquer l’emplacement des victimes|Suivre leurs instructions|Aucune des autres réponses|D</v>
+      </c>
+      <c r="D207" t="str" cm="1">
+        <f t="array" ref="D207:J207">_xlfn.TEXTSPLIT(C207,"|")</f>
+        <v>[UV7] Dès l’arrivée des forces de l’ordre, dans une zone d’attentat, vous devez en premier :</v>
+      </c>
+      <c r="E207" t="str">
+        <v>Leur parler de la situation</v>
+      </c>
+      <c r="F207" t="str">
+        <v>Courir vers eux</v>
+      </c>
+      <c r="G207" t="str">
+        <v>Leur indiquer l’emplacement des victimes</v>
+      </c>
+      <c r="H207" t="str">
+        <v>Suivre leurs instructions</v>
+      </c>
+      <c r="I207" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J207" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A208" s="18" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B208" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C208" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV7] Parmi les types de “BLAST” suivants, lequel ou lesquels existent ?|BLAST primaire|BLAST tertiaire|BLAST quaternaire|Toutes les réponses précédentes sont exactes|BLAST secondaire|D</v>
+      </c>
+      <c r="D208" t="str" cm="1">
+        <f t="array" ref="D208:J208">_xlfn.TEXTSPLIT(C208,"|")</f>
+        <v>[UV7] Parmi les types de “BLAST” suivants, lequel ou lesquels existent ?</v>
+      </c>
+      <c r="E208" t="str">
+        <v>BLAST primaire</v>
+      </c>
+      <c r="F208" t="str">
+        <v>BLAST tertiaire</v>
+      </c>
+      <c r="G208" t="str">
+        <v>BLAST quaternaire</v>
+      </c>
+      <c r="H208" t="str">
+        <v>Toutes les réponses précédentes sont exactes</v>
+      </c>
+      <c r="I208" t="str">
+        <v>BLAST secondaire</v>
+      </c>
+      <c r="J208" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A209" s="18" t="s">
+        <v>1249</v>
+      </c>
+      <c r="B209" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C209" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV2] Agent de sécurité, je dispose d’un véhicule d’entreprise équipé d’un gyrophare orange :|Aucune des autres réponses|C’est absolument interdit|C’est autorisé uniquement à l’intérieur des sites surveillés, si les consignes le prévoient|Seuls les gyrophares bleus sont autorisés pour les agents de sécurité|C’est interdit, sauf en situation d’urgence attentat|C</v>
+      </c>
+      <c r="D209" t="str" cm="1">
+        <f t="array" ref="D209:J209">_xlfn.TEXTSPLIT(C209,"|")</f>
+        <v>[UV2] Agent de sécurité, je dispose d’un véhicule d’entreprise équipé d’un gyrophare orange :</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="F209" t="str">
+        <v>C’est absolument interdit</v>
+      </c>
+      <c r="G209" t="str">
+        <v>C’est autorisé uniquement à l’intérieur des sites surveillés, si les consignes le prévoient</v>
+      </c>
+      <c r="H209" t="str">
+        <v>Seuls les gyrophares bleus sont autorisés pour les agents de sécurité</v>
+      </c>
+      <c r="I209" t="str">
+        <v>C’est interdit, sauf en situation d’urgence attentat</v>
+      </c>
+      <c r="J209" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A210" s="18" t="s">
+        <v>1250</v>
+      </c>
+      <c r="B210" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C210" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV2] Selon la loi, est une arme par destination :|Tout objet conçu pour usage professionnel|Tout objet conçu pour tuer ou blesser|Aucune des autres réponses|Tout objet susceptible de présenter un danger pour des personnes, dès lors qu’il est utilisé pour menacer|Tout objet pouvant causer des dommages|D</v>
+      </c>
+      <c r="D210" t="str" cm="1">
+        <f t="array" ref="D210:J210">_xlfn.TEXTSPLIT(C210,"|")</f>
+        <v>[UV2] Selon la loi, est une arme par destination :</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Tout objet conçu pour usage professionnel</v>
+      </c>
+      <c r="F210" t="str">
+        <v>Tout objet conçu pour tuer ou blesser</v>
+      </c>
+      <c r="G210" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="H210" t="str">
+        <v>Tout objet susceptible de présenter un danger pour des personnes, dès lors qu’il est utilisé pour menacer</v>
+      </c>
+      <c r="I210" t="str">
+        <v>Tout objet pouvant causer des dommages</v>
+      </c>
+      <c r="J210" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A211" s="18" t="s">
+        <v>1251</v>
+      </c>
+      <c r="B211" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C211" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV11] Le report d’alarme d’une centrale intrusion est un dispositif :|Uniquement destiné aux équipes de sûreté en cas d’intrusion|De secours en cas de défaillance du clavier principal|Qui permet aux agents d’accéder à certaines informations hors du PCS|De cloisonnement anti-intrusion indépendant du système central|Aucune des autres réponses|C</v>
+      </c>
+      <c r="D211" t="str" cm="1">
+        <f t="array" ref="D211:J211">_xlfn.TEXTSPLIT(C211,"|")</f>
+        <v>[UV11] Le report d’alarme d’une centrale intrusion est un dispositif :</v>
+      </c>
+      <c r="E211" t="str">
+        <v>Uniquement destiné aux équipes de sûreté en cas d’intrusion</v>
+      </c>
+      <c r="F211" t="str">
+        <v>De secours en cas de défaillance du clavier principal</v>
+      </c>
+      <c r="G211" t="str">
+        <v>Qui permet aux agents d’accéder à certaines informations hors du PCS</v>
+      </c>
+      <c r="H211" t="str">
+        <v>De cloisonnement anti-intrusion indépendant du système central</v>
+      </c>
+      <c r="I211" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J211" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A212" s="18" t="s">
+        <v>1252</v>
+      </c>
+      <c r="B212" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C212" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV14] Dans quel document l’APS peut trouver les mesures opératoires des secours extérieurs lors d’un sinistre majeur ?|Le Plan des Opérations Externes (P.O.E.)|Le Plan Particulier d’Intervention (P.P.I. ou équivalent)|Le Plan de Secours Extérieurs (P.S.E.)|Le Plan Particulier des Risques Majeurs (P.P.R.M.)|Aucune des autres réponses|B</v>
+      </c>
+      <c r="D212" t="str" cm="1">
+        <f t="array" ref="D212:J212">_xlfn.TEXTSPLIT(C212,"|")</f>
+        <v>[UV14] Dans quel document l’APS peut trouver les mesures opératoires des secours extérieurs lors d’un sinistre majeur ?</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Le Plan des Opérations Externes (P.O.E.)</v>
+      </c>
+      <c r="F212" t="str">
+        <v>Le Plan Particulier d’Intervention (P.P.I. ou équivalent)</v>
+      </c>
+      <c r="G212" t="str">
+        <v>Le Plan de Secours Extérieurs (P.S.E.)</v>
+      </c>
+      <c r="H212" t="str">
+        <v>Le Plan Particulier des Risques Majeurs (P.P.R.M.)</v>
+      </c>
+      <c r="I212" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J212" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A213" s="18" t="s">
+        <v>1253</v>
+      </c>
+      <c r="B213" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C213" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV14] Quand doit-on rédiger notamment impérativement un Plan de Prévention ?|En cas de travaux dangereux listés dans l’arrêté du 19 mars 1993|Uniquement lorsque les consignes de sûreté le prévoient|Si vous estimez que l’importance des travaux le nécessitent|Uniquement sur demande explicite du client|Aucune des autres réponses|A</v>
+      </c>
+      <c r="D213" t="str" cm="1">
+        <f t="array" ref="D213:J213">_xlfn.TEXTSPLIT(C213,"|")</f>
+        <v>[UV14] Quand doit-on rédiger notamment impérativement un Plan de Prévention ?</v>
+      </c>
+      <c r="E213" t="str">
+        <v>En cas de travaux dangereux listés dans l’arrêté du 19 mars 1993</v>
+      </c>
+      <c r="F213" t="str">
+        <v>Uniquement lorsque les consignes de sûreté le prévoient</v>
+      </c>
+      <c r="G213" t="str">
+        <v>Si vous estimez que l’importance des travaux le nécessitent</v>
+      </c>
+      <c r="H213" t="str">
+        <v>Uniquement sur demande explicite du client</v>
+      </c>
+      <c r="I213" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J213" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A214" s="18" t="s">
+        <v>1254</v>
+      </c>
+      <c r="B214" s="17">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="C214" s="17" t="str">
+        <f t="shared" si="23"/>
+        <v>[UV14] Quel est l’objectif général de la prévention ?|Définir les mesures de sûreté|Protéger l’employeur du risque pénal|Améliorer les statistiques concernant les taux d’accidents|Éviter ou limiter les dommages|Aucune des autres réponses|D</v>
+      </c>
+      <c r="D214" t="str" cm="1">
+        <f t="array" ref="D214:J214">_xlfn.TEXTSPLIT(C214,"|")</f>
+        <v>[UV14] Quel est l’objectif général de la prévention ?</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Définir les mesures de sûreté</v>
+      </c>
+      <c r="F214" t="str">
+        <v>Protéger l’employeur du risque pénal</v>
+      </c>
+      <c r="G214" t="str">
+        <v>Améliorer les statistiques concernant les taux d’accidents</v>
+      </c>
+      <c r="H214" t="str">
+        <v>Éviter ou limiter les dommages</v>
+      </c>
+      <c r="I214" t="str">
+        <v>Aucune des autres réponses</v>
+      </c>
+      <c r="J214" t="str">
+        <v>D</v>
       </c>
     </row>
   </sheetData>

</xml_diff>